<commit_message>
docs(us): bổ sung tiêu chí phi chức năng cho 75 US và thêm 15 US chất lượng
- Thêm 295 tiêu chí nghiệm thu phi chức năng vào 75 US sẵn có: hiển thị
  lỗi, trạng thái tải/rỗng, phân trang, xác nhận thao tác phá huỷ, thao
  tác bằng bàn phím, chống bấm lặp, responsive.
- Thêm 15 US cắt ngang (76-90) về chất lượng và trải nghiệm: chuẩn hoá
  lỗi, khung xương, phân trang, số đếm chưa đọc, a11y, màn hình nhỏ, mất
  kết nối realtime, giới hạn tần suất, bảo vệ dữ liệu trên trình duyệt.
- Tổng: 90 US / 742 tiêu chí nghiệm thu.

Hạ tầng dev cho kiểm thử: thêm MailHog vào docker-compose và trỏ SMTP
local về nó để email OTP không rời máy; mailer bỏ khối auth khi không có
thông tin đăng nhập (MailHog không dùng AUTH).
</commit_message>
<xml_diff>
--- a/docs/DALN-User-Stories.xlsx
+++ b/docs/DALN-User-Stories.xlsx
@@ -2,15 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="User Stories" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'User Stories'!$A$1:$F$76</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'User Stories'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,35 +28,32 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <family val="2"/>
+      <color rgb="FFffffff"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
+      <family val="2"/>
+      <color rgb="FFc0392b"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00C0392B"/>
+      <family val="2"/>
+      <color rgb="FFb9770e"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00B9770E"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="005D6D7E"/>
+      <family val="2"/>
+      <color rgb="FF5d6d7e"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -71,17 +66,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="005B7FE9"/>
+        <fgColor rgb="FF5b7fe9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E2D9"/>
+        <fgColor rgb="FFd9e2d9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF2E4"/>
+        <fgColor rgb="FFeaf2e4"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,66 +90,82 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="009FB3C8"/>
+        <color rgb="FF9fb3c8"/>
       </left>
       <right style="thin">
-        <color rgb="009FB3C8"/>
+        <color rgb="FF9fb3c8"/>
       </right>
       <top style="thin">
-        <color rgb="009FB3C8"/>
+        <color rgb="FF9fb3c8"/>
       </top>
       <bottom style="thin">
-        <color rgb="009FB3C8"/>
+        <color rgb="FF9fb3c8"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -233,10 +244,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -274,69 +285,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -360,54 +373,53 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -417,7 +429,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -426,7 +438,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -435,7 +447,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -443,10 +455,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -475,7 +487,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -488,13 +500,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
+                <a:tint val="80000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -514,258 +525,288 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="78" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="6.005" bestFit="1" customWidth="1" style="14" min="1" max="1"/>
+    <col width="26.005" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
+    <col width="58.005" bestFit="1" customWidth="1" style="15" min="3" max="3"/>
+    <col width="78.005" bestFit="1" customWidth="1" style="15" min="4" max="4"/>
+    <col width="10.005" bestFit="1" customWidth="1" style="16" min="5" max="5"/>
+    <col width="54.005" bestFit="1" customWidth="1" style="15" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="30" customFormat="1" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Module/ Epic</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>User Story</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="141" customHeight="1">
-      <c r="A2" s="2" t="n">
+    <row r="2" ht="330" customHeight="1">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Đăng ký tài khoản mới</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Là người dùng mới, tôi muốn đăng ký tài khoản bằng email, tên đăng nhập và mật khẩu, để tôi có danh tính riêng và bắt đầu sử dụng hệ thống trò chuyện.</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>- Người dùng nhập email, tên đăng nhập, mật khẩu và (tuỳ chọn) vị trí; hệ thống tạo tài khoản ở trạng thái chờ xác thực
 - Ngay sau khi đăng ký, hệ thống gửi mã OTP về email và chuyển người dùng sang màn hình nhập mã
 - Nếu email hoặc tên đăng nhập đã tồn tại, hệ thống báo lỗi rõ ràng và không tạo tài khoản trùng
 - Mật khẩu luôn được băm trước khi lưu, không bao giờ được trả về trong bất kỳ phản hồi nào
-- Tài khoản chưa xác thực OTP không thể đăng nhập vào ứng dụng</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
+- Tài khoản chưa xác thực OTP không thể đăng nhập vào ứng dụng
+- Biểu mẫu kiểm tra ngay khi rời khỏi từng ô: email sai định dạng, mật khẩu chưa đủ mạnh, tên đăng nhập quá ngắn đều báo lỗi ngay dưới ô đó, không đợi tới lúc bấm gửi
+- Ô mật khẩu có nút hiện/ẩn và thanh đo độ mạnh; nút gửi bị vô hiệu khi biểu mẫu chưa hợp lệ
+- Trong lúc gửi, nút chuyển sang trạng thái đang xử lý và không bấm lại được, tránh tạo trùng tài khoản do bấm nhiều lần
+- Lỗi trùng email hoặc trùng tên đăng nhập do máy chủ trả về được gắn vào đúng ô gây lỗi, không chỉ hiện thông báo nổi chung chung
+- Mất kết nối lúc gửi thì hiển thị thông báo không kết nối được máy chủ và giữ nguyên toàn bộ dữ liệu đã nhập trên biểu mẫu
+- Toàn bộ biểu mẫu thao tác được bằng bàn phím theo đúng thứ tự, mỗi ô có nhãn gắn đúng và lỗi được trình đọc màn hình đọc lên</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Đây là điểm khởi đầu của toàn bộ hành trình người dùng. Việc tách riêng bước tạo tài khoản và bước xác thực giúp đảm bảo mỗi tài khoản gắn với một email có thật, hạn chế tài khoản rác và tạo nền tảng tin cậy cho các tính năng xã hội phía sau.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="126" customHeight="1">
-      <c r="A3" s="2" t="n">
+    <row r="3" ht="315" customHeight="1">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Xác thực email bằng mã OTP</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Là người dùng vừa đăng ký, tôi muốn nhập mã OTP nhận được qua email, để kích hoạt tài khoản và chứng minh email đó thực sự thuộc về tôi.</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>- Người dùng nhập đúng mã OTP còn hiệu lực, hệ thống kích hoạt tài khoản và thông báo xác thực thành công
 - Nhập sai mã, hệ thống báo lỗi và cho phép thử lại mà không xoá dữ liệu đăng ký đã nhập
 - Mã OTP có thời hạn sử dụng; hết hạn thì không còn dùng được và người dùng phải yêu cầu mã mới
 - Một mã OTP chỉ dùng được một lần, sau khi xác thực thành công thì bị vô hiệu ngay
-- Sau khi xác thực thành công, người dùng được đưa về màn hình đăng nhập</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+- Sau khi xác thực thành công, người dùng được đưa về màn hình đăng nhập
+- Ô nhập mã tự chuyển ô khi gõ, hỗ trợ dán cả dãy số một lần và cho phép xoá lùi về ô trước
+- Màn hình hiển thị đồng hồ đếm ngược thời hạn còn lại của mã; hết giờ thì ô nhập bị khoá kèm hướng dẫn lấy mã mới
+- Trong lúc gửi mã đi kiểm tra, nút xác nhận hiển thị trạng thái đang xử lý và chặn bấm lặp
+- Nhập sai mã thì thông báo lỗi hiển thị ngay cạnh ô nhập và mã cũ được bôi chọn sẵn để gõ đè, không bắt người dùng tự xoá
+- Số lần nhập sai liên tiếp bị giới hạn; vượt ngưỡng thì tạm khoá thao tác kèm thông báo thời gian chờ
+- Truy cập màn hình xác thực mà thiếu tham số email thì hệ thống hướng người dùng quay lại bước đăng ký thay vì hiện màn hình hỏng</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Bước xác thực email bảo vệ hệ thống khỏi tài khoản giả mạo và đảm bảo kênh liên lạc dự phòng (email thông báo, email tổng hợp) luôn hoạt động cho từng người dùng.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="96" customHeight="1">
-      <c r="A4" s="2" t="n">
+    <row r="4" ht="225" customHeight="1">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Gửi lại mã OTP</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Là người dùng không nhận được email chứa mã OTP, tôi muốn yêu cầu gửi lại mã, để tôi không phải đăng ký lại từ đầu.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>- Người dùng bấm "Gửi lại mã", hệ thống phát hành mã OTP mới và gửi lại về đúng email đã đăng ký
 - Mã cũ bị vô hiệu ngay khi mã mới được phát hành
 - Hệ thống có khoảng chờ giữa hai lần gửi lại để tránh bị lạm dụng gửi thư hàng loạt
-- Nếu email không tồn tại trong danh sách chờ xác thực, hệ thống không tiết lộ thông tin đó mà chỉ trả về thông báo chung</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
+- Nếu email không tồn tại trong danh sách chờ xác thực, hệ thống không tiết lộ thông tin đó mà chỉ trả về thông báo chung
+- Nút gửi lại bị vô hiệu và hiển thị đồng hồ đếm ngược đúng số giây còn lại của khoảng chờ
+- Trạng thái đếm ngược vẫn đúng sau khi tải lại trang, người dùng không lách được khoảng chờ bằng cách làm mới trang
+- Gửi lại thành công thì hiện thông báo xác nhận đã gửi kèm địa chỉ email được che bớt, không lộ toàn bộ email
+- Khi máy chủ trả về lỗi giới hạn tần suất, giao diện hiển thị đúng thông điệp chờ thay vì lỗi kỹ thuật thô</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Email có thể vào thư mục spam hoặc bị chậm. Tính năng gửi lại giúp giảm tỷ lệ bỏ dở ở bước đăng ký, đồng thời vẫn kiểm soát được nguy cơ lạm dụng dịch vụ gửi thư.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="141" customHeight="1">
-      <c r="A5" s="2" t="n">
+    <row r="5" ht="330" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Đăng nhập vào hệ thống</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Là người dùng đã có tài khoản, tôi muốn đăng nhập bằng email và mật khẩu, để truy cập vào các cuộc trò chuyện và danh bạ bạn bè của mình.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>- Nhập đúng email và mật khẩu của tài khoản đã xác thực, hệ thống tạo phiên làm việc và đưa người dùng vào màn hình trò chuyện
 - Nhập sai thông tin, hệ thống hiển thị một thông báo lỗi chung, không cho biết sai email hay sai mật khẩu
 - Tài khoản chưa xác thực OTP bị từ chối đăng nhập kèm hướng dẫn hoàn tất xác thực
 - Thông tin phiên được lưu trong cookie chỉ đọc bởi máy chủ và truyền qua kênh mã hoá, không xuất hiện trên URL
-- Nếu người dùng chưa chọn sở thích lần nào, hệ thống chuyển sang màn hình chọn sở thích thay vì vào thẳng trò chuyện</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+- Nếu người dùng chưa chọn sở thích lần nào, hệ thống chuyển sang màn hình chọn sở thích thay vì vào thẳng trò chuyện
+- Trong lúc đăng nhập, nút hiển thị trạng thái đang xử lý và biểu mẫu bị khoá để chặn gửi lặp
+- Thông báo lỗi đăng nhập hiển thị cố định trên biểu mẫu (không chỉ là thông báo nổi tự tắt) để người dùng đọc kịp
+- Mật khẩu không bao giờ nằm trong lịch sử trình duyệt, URL hay bộ nhớ đệm; ô mật khẩu khai báo đúng thuộc tính để trình quản lý mật khẩu nhận diện
+- Nhấn Enter trong bất kỳ ô nào cũng gửi biểu mẫu, không bắt buộc phải bấm chuột vào nút
+- Số lần đăng nhập sai liên tiếp bị giới hạn để chống dò mật khẩu, kèm thông báo rõ ràng khi bị tạm khoá
+- Đăng nhập thành công thì mọi dữ liệu tạm của tài khoản trước đó trên trình duyệt được xoá trước khi nạp dữ liệu mới</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Đăng nhập là cổng vào duy nhất của ứng dụng. Việc trả về đầy đủ thông tin hồ sơ ngay tại bước này giúp giao diện dựng được ngay mà không cần gọi thêm, rút ngắn thời gian người dùng nhìn thấy nội dung.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="111" customHeight="1">
-      <c r="A6" s="2" t="n">
+    <row r="6" ht="240" customHeight="1">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Duy trì phiên đăng nhập</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Là người dùng đang sử dụng ứng dụng, tôi muốn phiên làm việc của mình được giữ và tự động gia hạn, để tôi không bị đăng xuất giữa chừng khi đang trò chuyện.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>- Khi tải lại trang, hệ thống tự khôi phục phiên từ cookie và lấy lại thông tin cá nhân mà không bắt đăng nhập lại
 - Khi phiên ngắn hạn hết hạn nhưng phiên dài hạn còn hiệu lực, hệ thống tự làm mới trong nền, người dùng không bị gián đoạn
 - Khi cả hai đều hết hạn hoặc bị thu hồi, hệ thống đưa người dùng về màn hình đăng nhập kèm thông báo phiên đã kết thúc
-- Mọi yêu cầu tới tài nguyên cần đăng nhập đều bị từ chối nếu phiên không hợp lệ</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+- Mọi yêu cầu tới tài nguyên cần đăng nhập đều bị từ chối nếu phiên không hợp lệ
+- Trong lúc khôi phục phiên, ứng dụng hiển thị màn hình chờ thay vì nháy qua màn hình đăng nhập rồi mới vào trong
+- Nhiều yêu cầu cùng hết hạn một lúc chỉ kích hoạt đúng một lần làm mới phiên, các yêu cầu còn lại chờ và được thử lại sau khi làm mới xong
+- Yêu cầu bị lỗi do phiên hết hạn được tự động gửi lại một lần sau khi làm mới thành công, người dùng không phải thao tác lại
+- Khi phiên bị thu hồi, ứng dụng dừng mọi vòng lặp gọi lại và không hiển thị hàng loạt thông báo lỗi chồng nhau</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Ứng dụng trò chuyện được mở liên tục trong nhiều giờ. Cơ chế gia hạn phiên tự động giữ trải nghiệm liền mạch trong khi vẫn giới hạn thời gian sống của thông tin xác thực để giảm rủi ro bảo mật.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="111" customHeight="1">
-      <c r="A7" s="2" t="n">
+    <row r="7" ht="225" customHeight="1">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Đăng xuất khỏi hệ thống</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn đăng xuất khỏi ứng dụng, để bảo vệ tài khoản khi dùng máy tính chung hoặc thiết bị không phải của mình.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>- Bấm đăng xuất, hệ thống xoá thông tin phiên khỏi trình duyệt và đưa người dùng về màn hình đăng nhập
 - Sau khi đăng xuất, mọi kết nối thời gian thực bị ngắt và trạng thái của người dùng chuyển sang ngoại tuyến
 - Bấm nút quay lại của trình duyệt không thể xem lại nội dung trò chuyện đã tải trước đó
-- Toàn bộ dữ liệu người dùng lưu tạm trên trình duyệt được dọn sạch</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+- Toàn bộ dữ liệu người dùng lưu tạm trên trình duyệt được dọn sạch
+- Nút đăng xuất hỏi xác nhận trước khi thực hiện để tránh bấm nhầm khi đang trò chuyện
+- Trong lúc đăng xuất, giao diện hiển thị trạng thái đang xử lý và chặn thao tác tiếp theo
+- Nếu yêu cầu đăng xuất tới máy chủ thất bại, ứng dụng vẫn dọn sạch phiên phía trình duyệt và đưa về màn hình đăng nhập
+- Sau khi đăng xuất, mở lại ứng dụng ở tab khác đang mở sẵn cũng bị đưa về màn hình đăng nhập</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Đăng xuất triệt để là yêu cầu cơ bản về quyền riêng tư, đặc biệt quan trọng với ứng dụng chứa nội dung trò chuyện cá nhân.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="111" customHeight="1">
-      <c r="A8" s="7" t="n">
+    <row r="8" ht="240" customHeight="1">
+      <c r="A8" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Chọn sở thích lần đầu</t>
         </is>
@@ -781,7 +822,12 @@
 - Người dùng phải chọn tối thiểu số lượng thẻ quy định mới có thể tiếp tục
 - Sau khi hoàn tất, hệ thống đánh dấu đã qua bước chọn sở thích và không hỏi lại ở các lần đăng nhập sau
 - Người dùng có thể bỏ qua và chỉnh lại sở thích sau trong phần hồ sơ
-- Sở thích đã chọn được dùng ngay cho lần tính gợi ý kết bạn kế tiếp</t>
+- Sở thích đã chọn được dùng ngay cho lần tính gợi ý kết bạn kế tiếp
+- Danh sách thẻ sở thích hiển thị khung xương trong lúc tải và hiển thị nút thử lại nếu tải thất bại
+- Bộ đếm số thẻ đã chọn và số tối thiểu còn thiếu luôn hiển thị; nút tiếp tục chỉ bật khi đã đủ
+- Thẻ sở thích chọn được bằng phím cách hoặc Enter khi di chuyển bằng bàn phím, trạng thái chọn được thông báo cho trình đọc màn hình
+- Trong lúc lưu, nút hiển thị trạng thái đang xử lý; lưu thất bại thì giữ nguyên các lựa chọn đã chọn và cho thử lại
+- Trên màn hình hẹp, lưới thẻ tự xuống dòng và không sinh thanh cuộn ngang</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -795,11 +841,11 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="81" customHeight="1">
-      <c r="A9" s="7" t="n">
+    <row r="9" ht="225" customHeight="1">
+      <c r="A9" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Xem hồ sơ cá nhân</t>
         </is>
@@ -814,7 +860,11 @@
           <t>- Hệ thống hiển thị tên hiển thị, tên đăng nhập, email, ảnh đại diện, giới thiệu bản thân và danh sách sở thích
 - Chỉ chủ tài khoản mới xem được email và các thông tin riêng tư của chính mình
 - Các trường chưa được điền hiển thị giá trị mặc định thay vì để trống gây khó hiểu
-- Thông tin luôn phản ánh dữ liệu mới nhất ngay sau khi người dùng cập nhật</t>
+- Thông tin luôn phản ánh dữ liệu mới nhất ngay sau khi người dùng cập nhật
+- Trong lúc tải hồ sơ, hệ thống hiển thị khung xương đúng bố cục thay vì màn hình trắng hoặc nội dung nhảy
+- Tải hồ sơ thất bại thì hiển thị thông báo lỗi kèm nút thử lại ngay trong bảng hồ sơ
+- Ảnh đại diện lỗi hoặc thiếu thì hiển thị chữ cái đầu của tên trên nền màu thay vì biểu tượng ảnh vỡ
+- Phần giới thiệu dài hoặc chuỗi ký tự liền không dấu cách vẫn xuống dòng, không đẩy vỡ bố cục</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -828,11 +878,11 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="156" customHeight="1">
-      <c r="A10" s="7" t="n">
+    <row r="10" ht="300" customHeight="1">
+      <c r="A10" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Cập nhật hồ sơ và ảnh đại diện</t>
         </is>
@@ -848,7 +898,12 @@
 - Ảnh đại diện được kiểm tra định dạng và kích thước trước khi chấp nhận, ảnh không hợp lệ bị từ chối kèm lý do
 - Ảnh đại diện mới được cập nhật đồng bộ tại danh sách bạn bè, danh sách hội thoại và tin nhắn cũ
 - Người dùng chỉ được sửa hồ sơ của chính mình, mọi yêu cầu sửa hồ sơ người khác đều bị từ chối
-- Nếu tải ảnh thất bại, các thông tin văn bản đã nhập vẫn được giữ nguyên trên biểu mẫu</t>
+- Nếu tải ảnh thất bại, các thông tin văn bản đã nhập vẫn được giữ nguyên trên biểu mẫu
+- Nút lưu chỉ bật khi có thay đổi thực sự; rời khỏi biểu mẫu khi còn thay đổi chưa lưu thì hệ thống hỏi xác nhận
+- Ảnh đại diện mới hiển thị xem trước ngay tại chỗ trước khi lưu, kèm nút huỷ chọn để quay lại ảnh cũ
+- Trong lúc tải ảnh lên, hệ thống hiển thị tiến độ và vô hiệu nút lưu để chặn gửi lặp
+- Giới hạn số ký tự của tên hiển thị và giới thiệu bản thân được thông báo trước bằng bộ đếm ký tự, không để người dùng gõ xong mới bị từ chối
+- Lưu thành công hiển thị thông báo xác nhận; lưu thất bại hiển thị lý do cụ thể và giữ nguyên nội dung đang sửa</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -862,11 +917,11 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="126" customHeight="1">
-      <c r="A11" s="7" t="n">
+    <row r="11" ht="240" customHeight="1">
+      <c r="A11" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Xem hồ sơ người dùng khác</t>
         </is>
@@ -881,7 +936,11 @@
           <t>- Bấm vào tên hoặc ảnh đại diện của một người, hệ thống mở bảng hồ sơ với tên hiển thị, ảnh, giới thiệu và sở thích
 - Bảng hồ sơ hiển thị đúng quan hệ hiện tại: chưa kết bạn, đã gửi lời mời, hoặc đã là bạn bè
 - Thông tin nhạy cảm như email và mật khẩu không bao giờ xuất hiện trong hồ sơ công khai
-- Nếu người dùng không tồn tại hoặc đã bị xoá, hệ thống hiển thị thông báo thay vì bảng trống</t>
+- Nếu người dùng không tồn tại hoặc đã bị xoá, hệ thống hiển thị thông báo thay vì bảng trống
+- Bảng hồ sơ mở ra hiển thị khung xương trong lúc tải và có thể đóng bằng phím Esc hoặc bấm ra ngoài
+- Nút hành động trên bảng hồ sơ phản ánh đúng quan hệ và chuyển sang trạng thái đang xử lý khi được bấm
+- Tiêu điểm bàn phím được chuyển vào bảng hồ sơ khi mở và trả về đúng phần tử đã bấm khi đóng
+- Tải hồ sơ thất bại thì hiển thị thông báo lỗi kèm nút thử lại thay vì bảng trống</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -895,214 +954,243 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="111" customHeight="1">
-      <c r="A12" s="2" t="n">
+    <row r="12" ht="270" customHeight="1">
+      <c r="A12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Tìm kiếm người dùng</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn tìm người khác theo tên hoặc tên đăng nhập, để chủ động tìm đúng người mình muốn kết nối.</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>- Người dùng nhập từ khoá, hệ thống trả về danh sách người dùng khớp kèm ảnh đại diện và trạng thái quan hệ
 - Kết quả tìm kiếm không bao gồm chính người đang tìm
 - Từ khoá rỗng hoặc quá ngắn thì không thực hiện tìm kiếm, tránh trả về toàn bộ danh bạ
 - Không có kết quả, hệ thống hiển thị thông báo rõ ràng thay vì danh sách trống
-- Kết quả chỉ chứa thông tin công khai, không lộ email hay dữ liệu cá nhân</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
+- Kết quả chỉ chứa thông tin công khai, không lộ email hay dữ liệu cá nhân
+- Ô tìm kiếm chờ người dùng ngừng gõ một khoảng ngắn rồi mới gọi máy chủ, tránh gọi liên tục theo từng ký tự
+- Kết quả của lần gõ cũ về sau kết quả mới thì bị bỏ qua, danh sách luôn khớp với từ khoá hiện tại
+- Trong lúc tìm, ô tìm kiếm hiển thị chỉ báo đang tải và giữ nguyên kết quả cũ thay vì nháy trắng
+- Kết quả tìm kiếm hỗ trợ tải thêm khi cuộn xuống, không giới hạn cứng ở nhóm kết quả đầu tiên
+- Ô tìm kiếm có nút xoá nhanh từ khoá và hỗ trợ phím Esc để xoá
+- Từ khoá có dấu tiếng Việt và khác biệt hoa thường vẫn cho ra cùng kết quả</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Tìm kiếm là con đường chủ động để mở rộng mạng lưới, bổ sung cho luồng gợi ý tự động. Đây là bước bắt buộc để người dùng có được người bạn đầu tiên.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="141" customHeight="1">
-      <c r="A13" s="2" t="n">
+    <row r="13" ht="255" customHeight="1">
+      <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Gửi lời mời kết bạn</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn gửi lời mời kết bạn tới một người, để bắt đầu xây dựng kết nối và có thể trò chuyện với họ.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>- Bấm "Kết bạn", hệ thống ghi nhận lời mời ở trạng thái chờ và cập nhật nút thành "Đã gửi lời mời"
 - Người nhận thấy thông báo lời mời mới ngay lập tức nếu đang trực tuyến, hoặc thấy khi mở ứng dụng lần sau
 - Không thể gửi lời mời tới chính mình, tới người đã là bạn, hoặc gửi trùng khi đã có lời mời đang chờ
 - Người dùng có thể kèm một lời nhắn ngắn khi gửi lời mời
-- Nếu người nhận đã gửi lời mời cho mình trước đó, hệ thống hướng dẫn chấp nhận thay vì tạo lời mời mới</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
+- Nếu người nhận đã gửi lời mời cho mình trước đó, hệ thống hướng dẫn chấp nhận thay vì tạo lời mời mới
+- Nút kết bạn chuyển sang trạng thái đang xử lý ngay khi bấm và không cho bấm lần hai trong lúc chờ
+- Kết quả thành công hoặc thất bại đều có phản hồi rõ ràng trên giao diện; thất bại thì nút trở lại trạng thái ban đầu để thử lại
+- Ô lời nhắn kèm theo có giới hạn ký tự kèm bộ đếm và loại bỏ khoảng trắng thừa trước khi gửi
+- Các trường hợp bị từ chối (tự kết bạn, đã là bạn, đã có lời mời chờ) hiển thị thông điệp riêng cho từng trường hợp thay vì một lỗi chung</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Lời mời kết bạn là cơ chế đồng thuận hai chiều, đảm bảo không ai bị thêm vào danh bạ người khác ngoài ý muốn. Đây là điều kiện tiên quyết để mở cuộc trò chuyện riêng tư.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="81" customHeight="1">
-      <c r="A14" s="2" t="n">
+    <row r="14" ht="255" customHeight="1">
+      <c r="A14" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Xem danh sách lời mời kết bạn</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn xem các lời mời kết bạn đã nhận và đã gửi, để nắm được ai đang chờ phản hồi của tôi và tôi đang chờ ai.</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>- Hệ thống hiển thị hai danh sách tách biệt: lời mời đã nhận và lời mời tôi đã gửi
 - Mỗi mục hiển thị ảnh đại diện, tên, lời nhắn kèm theo và thời điểm gửi
 - Danh sách hỗ trợ phân trang khi số lượng lời mời lớn
 - Lời mời đã được xử lý sẽ biến mất khỏi danh sách chờ ngay sau khi phản hồi
-- Người dùng chỉ xem được các lời mời liên quan trực tiếp tới mình</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
+- Người dùng chỉ xem được các lời mời liên quan trực tiếp tới mình
+- Mỗi tab hiển thị số lượng lời mời tương ứng ngay trên nhãn tab
+- Trang đầu tiên hiển thị khung xương trong lúc tải; các trang sau hiển thị chỉ báo tải thêm ở cuối danh sách
+- Phân trang không bao giờ lặp lại hay bỏ sót bản ghi khi có lời mời mới đến giữa lúc đang tải thêm
+- Đã tải hết danh sách thì nút tải thêm biến mất thay vì bấm được nhưng không có gì mới
+- Danh sách rỗng hiển thị trạng thái rỗng có hướng dẫn hành động tiếp theo, không phải vùng trắng
+- Tải danh sách thất bại thì hiển thị thông báo lỗi kèm nút thử lại ngay trong khu vực danh sách</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Tập trung mọi lời mời vào một nơi giúp người dùng không bỏ sót kết nối tiềm năng và hiểu rõ trạng thái từng quan hệ đang chờ.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="126" customHeight="1">
-      <c r="A15" s="2" t="n">
+    <row r="15" ht="255" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Chấp nhận hoặc từ chối lời mời kết bạn</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Là người nhận được lời mời, tôi muốn chấp nhận hoặc từ chối, để tự quyết định ai được vào danh sách bạn bè của mình.</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>- Chấp nhận lời mời, hai người trở thành bạn bè và hệ thống tự tạo sẵn một cuộc trò chuyện riêng giữa hai người
 - Người gửi nhận được thông báo kết quả ngay lập tức, danh sách bạn bè hai phía cùng được cập nhật
 - Từ chối lời mời, quan hệ không được tạo và lời mời rời khỏi danh sách chờ
 - Chỉ người nhận mới có quyền phản hồi lời mời; người khác thao tác đều bị từ chối
-- Nếu một bước trong quá trình xử lý thất bại, hệ thống hoàn tác toàn bộ, không để tồn tại quan hệ bạn bè mà thiếu cuộc trò chuyện</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+- Nếu một bước trong quá trình xử lý thất bại, hệ thống hoàn tác toàn bộ, không để tồn tại quan hệ bạn bè mà thiếu cuộc trò chuyện
+- Hai nút chấp nhận và từ chối đều chuyển sang trạng thái đang xử lý và khoá lẫn nhau trong lúc chờ máy chủ
+- Giao diện cập nhật lạc quan ngay khi bấm và tự hoàn nguyên đúng trạng thái cũ nếu máy chủ báo lỗi
+- Từ chối lời mời hỏi xác nhận trước khi thực hiện vì thao tác không hoàn tác được
+- Lời mời đã bị người khác xử lý trước đó (bấm lại từ tab cũ) hiển thị thông báo lời mời không còn hiệu lực thay vì lỗi kỹ thuật</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Đây là thao tác thay đổi dữ liệu ở nhiều dịch vụ cùng lúc: quan hệ bạn bè, cuộc trò chuyện và thông báo. Yêu cầu trọn vẹn hoặc không gì cả là điều kiện bắt buộc để dữ liệu không rơi vào trạng thái nửa vời.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="96" customHeight="1">
-      <c r="A16" s="2" t="n">
+    <row r="16" ht="255" customHeight="1">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Xem danh sách bạn bè</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn xem toàn bộ bạn bè của mình kèm trạng thái trực tuyến, để biết ai đang sẵn sàng trò chuyện.</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>- Hệ thống hiển thị danh sách bạn bè kèm ảnh đại diện, tên và dấu hiệu trực tuyến hay ngoại tuyến
 - Bạn bè đang trực tuyến được ưu tiên hiển thị hoặc đánh dấu nổi bật
 - Danh sách hỗ trợ phân trang và tìm kiếm nhanh theo tên
 - Bấm vào một người bạn sẽ mở ngay cuộc trò chuyện với người đó
-- Khi chưa có bạn nào, hệ thống hiển thị gợi ý kết bạn thay vì màn hình trống</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
+- Khi chưa có bạn nào, hệ thống hiển thị gợi ý kết bạn thay vì màn hình trống
+- Ô tìm nhanh trong danh sách bạn bè lọc tại chỗ, có nút xoá từ khoá và trạng thái không tìm thấy riêng
+- Danh sách dài dùng tải thêm theo trang, không tải toàn bộ trong một lần gọi
+- Trong lúc tải trang đầu, danh sách hiển thị khung xương giữ đúng chiều cao để bố cục không nhảy
+- Trạng thái trực tuyến có cả dấu hiệu bằng chữ, không chỉ dựa vào màu sắc của chấm tròn
+- Danh sách di chuyển được bằng phím mũi tên và mở cuộc trò chuyện bằng Enter</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Danh sách bạn bè là điểm xuất phát của mọi cuộc trò chuyện. Gắn trạng thái trực tuyến trực tiếp vào danh sách giúp người dùng chọn đúng thời điểm để bắt chuyện.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="126" customHeight="1">
-      <c r="A17" s="2" t="n">
+    <row r="17" ht="225" customHeight="1">
+      <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Nhận cập nhật kết bạn theo thời gian thực</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Là người dùng đang mở ứng dụng, tôi muốn thấy ngay khi có lời mời mới hoặc khi lời mời của tôi được phản hồi, để không phải tải lại trang mới biết.</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>- Khi có người gửi lời mời, biểu tượng thông báo và danh sách lời mời của người nhận tự cập nhật ngay
 - Khi lời mời được chấp nhận hoặc từ chối, người gửi thấy trạng thái đổi ngay mà không cần thao tác gì
 - Nếu người dùng đang ngoại tuyến, các thay đổi được hiển thị đầy đủ ở lần mở ứng dụng kế tiếp
-- Khi mất kết nối tạm thời, hệ thống tự kết nối lại và đồng bộ những thay đổi bị bỏ lỡ</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
+- Khi mất kết nối tạm thời, hệ thống tự kết nối lại và đồng bộ những thay đổi bị bỏ lỡ
+- Khi mất kết nối thời gian thực, giao diện hiển thị dải thông báo mất kết nối và tự ẩn khi kết nối lại
+- Sau khi kết nối lại, ứng dụng tự tải lại danh sách lời mời và số đếm để bù các thay đổi bị bỏ lỡ
+- Cùng một sự kiện đến hai lần không tạo hai mục trùng nhau trong danh sách
+- Cập nhật thời gian thực không làm mất vị trí cuộn hoặc thao tác đang dở của người dùng</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Phản hồi tức thời khiến trải nghiệm kết bạn trở nên sống động như một mạng xã hội thật, thay vì cảm giác thao tác trên một biểu mẫu tĩnh.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="111" customHeight="1">
-      <c r="A18" s="7" t="n">
+    <row r="18" ht="240" customHeight="1">
+      <c r="A18" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Tạo cuộc trò chuyện 1-1</t>
         </is>
@@ -1118,7 +1206,11 @@
 - Nếu hai người đã có cuộc trò chuyện riêng trước đó, hệ thống mở lại đúng cuộc trò chuyện cũ kèm toàn bộ lịch sử thay vì tạo mới
 - Chỉ hai thành viên trong cuộc trò chuyện riêng mới đọc được nội dung bên trong
 - Cuộc trò chuyện mới xuất hiện ngay trên danh sách hội thoại của cả hai phía
-- Không thể tạo cuộc trò chuyện riêng với người chưa phải là bạn bè</t>
+- Không thể tạo cuộc trò chuyện riêng với người chưa phải là bạn bè
+- Trong lúc mở hoặc tạo cuộc trò chuyện, giao diện hiển thị trạng thái đang mở thay vì khung chat trống
+- Bấm nhiều lần liên tiếp vào nút nhắn tin chỉ tạo đúng một cuộc trò chuyện
+- Mở cuộc trò chuyện thất bại thì hiển thị thông báo lỗi kèm nút thử lại, không để khung chat trắng
+- Đường dẫn cuộc trò chuyện trên trình duyệt mở lại được trực tiếp và giữ đúng cuộc trò chuyện sau khi tải lại trang</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -1132,11 +1224,11 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="111" customHeight="1">
-      <c r="A19" s="7" t="n">
+    <row r="19" ht="300" customHeight="1">
+      <c r="A19" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Tạo nhóm trò chuyện</t>
         </is>
@@ -1152,7 +1244,12 @@
 - Tất cả thành viên được chọn nhìn thấy nhóm mới trên danh sách hội thoại của họ ngay lập tức
 - Nhóm phải có tên và ít nhất hai thành viên ngoài người tạo mới được tạo thành công
 - Người dùng có thể đặt ảnh đại diện cho nhóm, nếu không hệ thống dùng ảnh mặc định
-- Một tin nhắn hệ thống ghi nhận sự kiện nhóm được tạo xuất hiện đầu cuộc trò chuyện</t>
+- Một tin nhắn hệ thống ghi nhận sự kiện nhóm được tạo xuất hiện đầu cuộc trò chuyện
+- Biểu mẫu tạo nhóm kiểm tra ngay tại chỗ: thiếu tên nhóm hoặc chưa đủ số thành viên tối thiểu đều báo lỗi dưới đúng trường
+- Danh sách bạn bè trong biểu mẫu có ô tìm kiếm, hiển thị số người đã chọn và cho bỏ chọn nhanh
+- Trong lúc tạo, nút tạo hiển thị trạng thái đang xử lý và chặn bấm lặp để không tạo hai nhóm trùng
+- Tạo nhóm thất bại thì giữ nguyên tên nhóm và danh sách đã chọn để người dùng thử lại
+- Ảnh nhóm được kiểm tra định dạng và dung lượng ngay khi chọn, kèm xem trước trước khi tạo</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -1166,11 +1263,11 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="111" customHeight="1">
-      <c r="A20" s="7" t="n">
+    <row r="20" ht="300" customHeight="1">
+      <c r="A20" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>Xem danh sách cuộc trò chuyện</t>
         </is>
@@ -1186,7 +1283,13 @@
 - Cuộc trò chuyện có tin nhắn mới nhất luôn được đẩy lên đầu danh sách ngay khi tin nhắn tới
 - Cuộc trò chuyện có tin chưa đọc được đánh dấu nổi bật kèm số lượng tin chưa đọc
 - Danh sách tải theo từng trang khi người dùng cuộn xuống, không tải toàn bộ một lần
-- Người dùng chỉ nhìn thấy các cuộc trò chuyện mà mình là thành viên</t>
+- Người dùng chỉ nhìn thấy các cuộc trò chuyện mà mình là thành viên
+- Danh sách hội thoại tải thêm theo con trỏ khi cuộn xuống, kèm chỉ báo đang tải ở cuối danh sách
+- Con trỏ phân trang xử lý đúng các cuộc trò chuyện có cùng mốc thời gian, không lặp lại hay bỏ sót mục
+- Trong lúc tải trang đầu, danh sách hiển thị khung xương thay vì vùng trắng
+- Trích đoạn tin nhắn cuối được cắt gọn trên một dòng và hiển thị đúng nhãn cho tin nhắn có tệp đính kèm hoặc bình chọn
+- Cuộc trò chuyện đang mở được đánh dấu rõ trong danh sách và giữ nguyên khi danh sách sắp xếp lại
+- Khi chưa có cuộc trò chuyện nào, danh sách hiển thị trạng thái rỗng kèm nút bắt đầu trò chuyện mới</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -1200,11 +1303,11 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="111" customHeight="1">
-      <c r="A21" s="7" t="n">
+    <row r="21" ht="225" customHeight="1">
+      <c r="A21" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Xem thông tin chi tiết cuộc trò chuyện</t>
         </is>
@@ -1219,7 +1322,11 @@
           <t>- Mở bảng thông tin, hệ thống hiển thị tên, ảnh đại diện, loại cuộc trò chuyện và toàn bộ thành viên kèm vai trò
 - Vai trò chủ nhóm và quản trị viên được đánh dấu rõ để phân biệt với thành viên thường
 - Bảng thông tin có lối đi nhanh tới kho ảnh, tệp và liên kết đã chia sẻ trong cuộc trò chuyện
-- Người không phải thành viên truy cập vào cuộc trò chuyện đều bị từ chối</t>
+- Người không phải thành viên truy cập vào cuộc trò chuyện đều bị từ chối
+- Bảng thông tin mở và đóng được bằng bàn phím, tiêu điểm bị giữ trong bảng khi đang mở
+- Danh sách thành viên đông người được cuộn riêng trong bảng và có ô tìm nhanh theo tên
+- Trong lúc tải, bảng hiển thị khung xương; tải thất bại thì hiển thị lỗi kèm nút thử lại
+- Trên màn hình hẹp, bảng thông tin hiển thị dạng lớp phủ toàn màn hình thay vì cột bị bóp méo</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1233,11 +1340,11 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="111" customHeight="1">
-      <c r="A22" s="7" t="n">
+    <row r="22" ht="210" customHeight="1">
+      <c r="A22" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Tìm kiếm cuộc trò chuyện và tin nhắn</t>
         </is>
@@ -1252,7 +1359,11 @@
           <t>- Nhập từ khoá, hệ thống trả về các cuộc trò chuyện có tên nhóm hoặc tên thành viên khớp
 - Kết quả hiển thị kèm ngữ cảnh đủ để người dùng nhận ra đúng cuộc trò chuyện cần tìm
 - Không có kết quả, hệ thống hiển thị thông báo rõ ràng
-- Kết quả tìm kiếm chỉ giới hạn trong các cuộc trò chuyện mà người dùng là thành viên</t>
+- Kết quả tìm kiếm chỉ giới hạn trong các cuộc trò chuyện mà người dùng là thành viên
+- Ô tìm kiếm chờ ngừng gõ rồi mới gọi máy chủ và huỷ kết quả của lần gõ cũ
+- Từ khoá khớp được làm nổi bật trong kết quả để người dùng thấy vì sao mục đó xuất hiện
+- Kết quả hiển thị chỉ báo đang tải và có thể xoá nhanh từ khoá để quay lại danh sách đầy đủ
+- Tìm kiếm thất bại thì hiển thị thông báo lỗi kèm nút thử lại thay vì trạng thái không có kết quả gây hiểu nhầm</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -1266,11 +1377,11 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="96" customHeight="1">
-      <c r="A23" s="7" t="n">
+    <row r="23" ht="210" customHeight="1">
+      <c r="A23" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Xoá lịch sử trò chuyện phía tôi</t>
         </is>
@@ -1285,7 +1396,11 @@
           <t>- Bấm xoá lịch sử, hệ thống hỏi xác nhận trước khi thực hiện vì thao tác không thể hoàn tác
 - Sau khi xác nhận, khung trò chuyện của người dùng trống nhưng cuộc trò chuyện vẫn còn trong danh sách
 - Các thành viên khác vẫn nhìn thấy đầy đủ lịch sử tin nhắn của họ
-- Tin nhắn mới gửi sau thời điểm xoá vẫn hiển thị bình thường với người dùng</t>
+- Tin nhắn mới gửi sau thời điểm xoá vẫn hiển thị bình thường với người dùng
+- Hộp thoại xác nhận nêu rõ hậu quả và yêu cầu thao tác chủ động, nút xác nhận dùng kiểu cảnh báo
+- Trong lúc xoá, nút xác nhận hiển thị trạng thái đang xử lý và không bấm lặp được
+- Xoá thất bại thì lịch sử giữ nguyên và hệ thống báo lỗi rõ ràng, không để khung chat trống nhầm
+- Sau khi xoá, khung chat hiển thị trạng thái rỗng có hướng dẫn thay vì vùng trắng không giải thích</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1299,11 +1414,11 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="111" customHeight="1">
-      <c r="A24" s="7" t="n">
+    <row r="24" ht="225" customHeight="1">
+      <c r="A24" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Xoá cuộc trò chuyện</t>
         </is>
@@ -1318,7 +1433,11 @@
           <t>- Bấm xoá, hệ thống hỏi xác nhận rồi gỡ cuộc trò chuyện khỏi danh sách của người dùng
 - Với nhóm, người dùng bị coi là đã rời nhóm và không nhận thêm tin nhắn mới từ nhóm đó
 - Các thành viên còn lại vẫn tiếp tục trò chuyện bình thường
-- Nếu sau này có người nhắn tin riêng lại, cuộc trò chuyện được khôi phục trong danh sách</t>
+- Nếu sau này có người nhắn tin riêng lại, cuộc trò chuyện được khôi phục trong danh sách
+- Hộp thoại xác nhận phân biệt rõ xoá cuộc trò chuyện riêng và rời nhóm, nêu đúng hậu quả từng loại
+- Sau khi xoá, hệ thống chuyển người dùng về danh sách hội thoại thay vì để lại khung chat của cuộc trò chuyện vừa xoá
+- Xoá thất bại thì cuộc trò chuyện được đưa trở lại danh sách kèm thông báo lỗi
+- Thao tác xoá có sẵn trong trình đơn ngữ cảnh của từng mục danh sách, không bắt buộc phải mở cuộc trò chuyện mới xoá được</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
@@ -1332,146 +1451,162 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="126" customHeight="1">
-      <c r="A25" s="2" t="n">
+    <row r="25" ht="255" customHeight="1">
+      <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>Thêm thành viên vào nhóm</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Là chủ nhóm hoặc quản trị viên, tôi muốn thêm bạn bè vào nhóm hiện có, để mở rộng nhóm khi cần thêm người tham gia.</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>- Chủ nhóm hoặc quản trị viên chọn thêm thành viên, người được thêm xuất hiện ngay trong danh sách thành viên
 - Người được thêm nhìn thấy nhóm mới trên danh sách hội thoại của họ ngay lập tức
 - Thành viên thường không có quyền thêm người, nút thao tác bị ẩn và yêu cầu bị từ chối ở phía máy chủ
 - Không thể thêm người đã là thành viên của nhóm
-- Một tin nhắn hệ thống ghi nhận ai đã thêm ai vào nhóm được hiển thị cho mọi thành viên</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
+- Một tin nhắn hệ thống ghi nhận ai đã thêm ai vào nhóm được hiển thị cho mọi thành viên
+- Hộp thoại thêm thành viên có ô tìm kiếm, ẩn sẵn những người đã ở trong nhóm và hiển thị số người đang chọn
+- Trong lúc thêm, nút xác nhận hiển thị trạng thái đang xử lý; thêm thất bại thì giữ nguyên lựa chọn để thử lại
+- Kết quả trả về phân biệt rõ người thêm thành công và người thất bại khi thêm nhiều người cùng lúc
+- Danh sách bạn bè trong hộp thoại tải thêm khi cuộn, không giới hạn ở nhóm đầu tiên</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>Nhóm là thực thể sống, thành phần thay đổi theo thời gian. Ràng buộc quyền theo vai trò ngăn nhóm bị thêm người tuỳ tiện, giữ được sự tin cậy trong không gian riêng của nhóm.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="126" customHeight="1">
-      <c r="A26" s="2" t="n">
+    <row r="26" ht="240" customHeight="1">
+      <c r="A26" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Xoá thành viên khỏi nhóm</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Là chủ nhóm hoặc quản trị viên, tôi muốn loại một thành viên khỏi nhóm, để xử lý trường hợp tham gia nhầm hoặc vi phạm.</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>- Chủ nhóm hoặc quản trị viên chọn xoá, thành viên bị loại khỏi danh sách và không nhận thêm tin nhắn của nhóm
 - Nhóm biến mất khỏi danh sách hội thoại của người bị loại ngay lập tức
 - Thành viên thường không thể loại người khác; chủ nhóm không thể bị loại bởi quản trị viên
 - Lịch sử tin nhắn cũ mà người bị loại đã gửi vẫn được giữ nguyên trong nhóm
-- Một tin nhắn hệ thống ghi nhận việc loại thành viên được hiển thị cho các thành viên còn lại</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
+- Một tin nhắn hệ thống ghi nhận việc loại thành viên được hiển thị cho các thành viên còn lại
+- Thao tác xoá thành viên hỏi xác nhận kèm tên người bị xoá để tránh bấm nhầm dòng
+- Trong lúc xử lý, dòng thành viên đó hiển thị trạng thái đang xử lý; thất bại thì hoàn nguyên và báo lỗi
+- Nút xoá bị ẩn hoàn toàn với người không đủ quyền thay vì hiện rồi báo lỗi khi bấm
+- Danh sách thành viên tự cập nhật số lượng ngay sau khi xoá thành công, không cần đóng mở lại bảng</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Khả năng loại thành viên là công cụ kiểm duyệt tối thiểu cho người quản lý nhóm, đồng thời phân cấp quyền ngăn việc lạm dụng loại trừ lẫn nhau.</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="126" customHeight="1">
-      <c r="A27" s="2" t="n">
+    <row r="27" ht="240" customHeight="1">
+      <c r="A27" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>Rời khỏi nhóm</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Là thành viên của một nhóm, tôi muốn tự rời nhóm, để không tiếp tục nhận nội dung mà tôi không còn quan tâm.</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>- Bấm rời nhóm, hệ thống hỏi xác nhận rồi gỡ người dùng khỏi danh sách thành viên
 - Sau khi rời, người dùng không còn nhận tin nhắn mới và nhóm biến mất khỏi danh sách hội thoại của họ
 - Khi chủ nhóm rời đi, hệ thống chuyển quyền chủ nhóm cho một thành viên còn lại thay vì để nhóm không có người quản lý
 - Một tin nhắn hệ thống ghi nhận việc rời nhóm được hiển thị cho các thành viên còn lại
-- Người đã rời có thể được mời lại vào nhóm sau này</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
+- Người đã rời có thể được mời lại vào nhóm sau này
+- Hộp thoại xác nhận rời nhóm nêu rõ hậu quả và trường hợp đặc biệt khi người rời là chủ nhóm
+- Trong lúc rời, nút xác nhận hiển thị trạng thái đang xử lý và chặn bấm lặp
+- Rời nhóm thất bại thì người dùng vẫn ở trong nhóm và nhận thông báo lỗi rõ ràng
+- Sau khi rời thành công, hệ thống chuyển về danh sách hội thoại kèm thông báo xác nhận</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>Quyền tự rời khỏi một không gian chung là yêu cầu cơ bản về sự tự chủ của người dùng. Xử lý trường hợp chủ nhóm rời đi tránh để nhóm rơi vào trạng thái không ai quản lý được.</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="111" customHeight="1">
-      <c r="A28" s="2" t="n">
+    <row r="28" ht="210" customHeight="1">
+      <c r="A28" s="4" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Theo dõi thay đổi thành viên theo thời gian thực</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Là thành viên trong nhóm, tôi muốn thấy ngay khi có người được thêm, bị loại hoặc rời nhóm, để luôn nắm được nhóm đang gồm những ai.</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>- Mọi thay đổi thành viên đều sinh một tin nhắn hệ thống hiển thị đúng vị trí thời gian trong dòng trò chuyện
 - Danh sách thành viên và số lượng thành viên tự cập nhật cho tất cả người đang mở nhóm
 - Người dùng đang ngoại tuyến sẽ thấy đầy đủ các tin nhắn hệ thống này khi mở lại nhóm
-- Tin nhắn hệ thống không thể bị chỉnh sửa hay thu hồi bởi bất kỳ ai</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
+- Tin nhắn hệ thống không thể bị chỉnh sửa hay thu hồi bởi bất kỳ ai
+- Tin nhắn hệ thống có kiểu hiển thị riêng, phân biệt rõ với tin nhắn của người dùng và không có ảnh đại diện
+- Nhiều thay đổi thành viên liên tiếp được gộp hiển thị gọn thay vì đẩy một chuỗi dài tin nhắn hệ thống
+- Cùng một sự kiện đến hai lần chỉ hiển thị một tin nhắn hệ thống
+- Tin nhắn hệ thống đến khi người dùng đang cuộn đọc tin cũ thì không tự kéo màn hình xuống dưới</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>Ghi nhận minh bạch các thay đổi thành viên xây dựng lòng tin trong nhóm, giúp mọi người biết chính xác ai có thể đọc được nội dung mình vừa chia sẻ.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="126" customHeight="1">
-      <c r="A29" s="7" t="n">
+    <row r="29" ht="285" customHeight="1">
+      <c r="A29" s="8" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Gửi tin nhắn văn bản tức thời</t>
         </is>
@@ -1487,7 +1622,13 @@
 - Khi máy chủ xác nhận đã lưu, tin nhắn chuyển sang trạng thái đã gửi kèm thời gian chính thức
 - Tin nhắn rỗng hoặc chỉ chứa khoảng trắng không được gửi đi
 - Mỗi tin nhắn mang một mã do máy khách sinh ra, gửi lại nhiều lần cũng không tạo tin nhắn trùng lặp
-- Người không phải thành viên cuộc trò chuyện không thể gửi tin nhắn vào đó</t>
+- Người không phải thành viên cuộc trò chuyện không thể gửi tin nhắn vào đó
+- Ô soạn tin tự giãn theo nội dung tới một chiều cao tối đa rồi mới cuộn bên trong
+- Enter gửi tin, Shift+Enter xuống dòng; quy ước này áp dụng nhất quán trên toàn ứng dụng
+- Nội dung đang gõ dở của mỗi cuộc trò chuyện được giữ lại khi chuyển sang cuộc trò chuyện khác rồi quay lại
+- Độ dài tin nhắn có giới hạn rõ ràng, hiển thị bộ đếm khi gần chạm ngưỡng và chặn gửi khi vượt
+- Sau khi gửi, tiêu điểm vẫn ở ô soạn tin để người dùng gõ tiếp ngay mà không phải bấm chuột
+- Khung chat tự cuộn xuống tin mới nhất khi chính người dùng gửi tin</t>
         </is>
       </c>
       <c r="E29" s="11" t="inlineStr">
@@ -1501,11 +1642,11 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="141" customHeight="1">
-      <c r="A30" s="7" t="n">
+    <row r="30" ht="255" customHeight="1">
+      <c r="A30" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Nhận tin nhắn theo thời gian thực</t>
         </is>
@@ -1521,7 +1662,11 @@
 - Nếu người dùng đang ở cuộc trò chuyện khác, hệ thống cập nhật trích đoạn và số tin chưa đọc trên danh sách hội thoại
 - Khi mất kết nối rồi kết nối lại, các tin nhắn bị bỏ lỡ được tải bổ sung và sắp đúng thứ tự thời gian
 - Tin nhắn chỉ được gửi tới đúng các thành viên của cuộc trò chuyện
-- Người dùng đăng nhập trên nhiều thiết bị đều nhận được tin nhắn trên tất cả thiết bị</t>
+- Người dùng đăng nhập trên nhiều thiết bị đều nhận được tin nhắn trên tất cả thiết bị
+- Khi người dùng đang cuộn đọc tin cũ, tin nhắn mới đến không kéo màn hình xuống mà hiển thị nút nhảy tới tin mới nhất kèm số tin chưa xem
+- Tin nhắn đến trùng với tin đã hiển thị (do gửi lại sự kiện) không sinh bản trùng trên giao diện
+- Khung chat tải nhiều tin nhắn vẫn giữ được độ mượt khi cuộn, không giật khi danh sách dài
+- Tin nhắn của chính người dùng đến qua kênh thời gian thực được ghép với tin nhắn tạm đang hiển thị thay vì thêm bản mới</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
@@ -1535,11 +1680,11 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="111" customHeight="1">
-      <c r="A31" s="7" t="n">
+    <row r="31" ht="285" customHeight="1">
+      <c r="A31" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Tải lịch sử tin nhắn</t>
         </is>
@@ -1555,7 +1700,12 @@
 - Cuộn lên đầu danh sách, hệ thống tự tải thêm nhóm tin nhắn cũ hơn kèm chỉ báo đang tải
 - Vị trí cuộn được giữ nguyên sau khi tải thêm, người dùng không bị nhảy màn hình
 - Khi đã tải hết lịch sử, hệ thống báo đã đến đầu cuộc trò chuyện và ngừng tải thêm
-- Chỉ thành viên của cuộc trò chuyện mới đọc được lịch sử tin nhắn</t>
+- Chỉ thành viên của cuộc trò chuyện mới đọc được lịch sử tin nhắn
+- Chỉ báo đang tải tin cũ hiển thị ở đầu danh sách và không che mất nội dung tin nhắn
+- Con trỏ phân trang xử lý đúng các tin nhắn có cùng mốc thời gian, không lặp lại hay bỏ sót tin
+- Cuộn nhanh liên tục không kích hoạt nhiều lần tải chồng nhau cho cùng một trang
+- Tải tin cũ thất bại thì hiển thị thông báo lỗi kèm nút thử lại ngay tại đầu danh sách
+- Tin nhắn được nhóm theo ngày với dải phân cách ngày dính ở đầu khung nhìn khi cuộn</t>
         </is>
       </c>
       <c r="E31" s="11" t="inlineStr">
@@ -1569,11 +1719,11 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="111" customHeight="1">
-      <c r="A32" s="7" t="n">
+    <row r="32" ht="225" customHeight="1">
+      <c r="A32" s="8" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Trả lời một tin nhắn cụ thể</t>
         </is>
@@ -1589,7 +1739,11 @@
 - Tin nhắn gửi đi hiển thị kèm trích dẫn tin nhắn gốc cho tất cả thành viên
 - Bấm vào phần trích dẫn sẽ cuộn tới đúng vị trí tin nhắn gốc trong lịch sử
 - Nếu tin nhắn gốc đã bị thu hồi, phần trích dẫn hiển thị trạng thái tin nhắn đã bị thu hồi
-- Người dùng có thể huỷ trả lời trước khi gửi mà không mất nội dung đang gõ</t>
+- Người dùng có thể huỷ trả lời trước khi gửi mà không mất nội dung đang gõ
+- Khung trích dẫn trong ô soạn thảo hiển thị tên người gửi và nội dung rút gọn, có nút huỷ và đóng được bằng phím Esc
+- Nhảy tới tin nhắn gốc có hiệu ứng làm nổi bật tạm thời để người dùng nhận ra vị trí
+- Tin nhắn gốc chưa được tải về thì hệ thống tự tải phần lịch sử cần thiết trước khi cuộn tới
+- Tin nhắn gốc đã bị xoá ở phía người dùng thì trích dẫn hiển thị trạng thái không còn khả dụng thay vì báo lỗi</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -1603,11 +1757,11 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="96" customHeight="1">
-      <c r="A33" s="7" t="n">
+    <row r="33" ht="210" customHeight="1">
+      <c r="A33" s="8" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Thu hồi tin nhắn đã gửi</t>
         </is>
@@ -1623,7 +1777,11 @@
 - Thay đổi được đẩy tới mọi thành viên đang mở cuộc trò chuyện ngay lập tức
 - Chỉ người gửi mới có quyền thu hồi tin nhắn của chính mình
 - Nội dung và tệp đính kèm gốc không còn được trả về cho bất kỳ ai sau khi thu hồi
-- Tin nhắn hệ thống không thể bị thu hồi</t>
+- Tin nhắn hệ thống không thể bị thu hồi
+- Thao tác thu hồi hỏi xác nhận và nêu rõ là không thể hoàn tác
+- Trong lúc thu hồi, tin nhắn hiển thị trạng thái đang xử lý; thất bại thì hoàn nguyên và báo lỗi
+- Tin nhắn đã thu hồi vẫn giữ đúng vị trí thời gian trong dòng trò chuyện, không làm xáo trộn thứ tự
+- Trích đoạn của cuộc trò chuyện trên danh sách hội thoại cũng được cập nhật khi tin nhắn cuối bị thu hồi</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -1637,11 +1795,11 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="81" customHeight="1">
-      <c r="A34" s="7" t="n">
+    <row r="34" ht="180" customHeight="1">
+      <c r="A34" s="8" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Xoá tin nhắn chỉ ở phía tôi</t>
         </is>
@@ -1656,7 +1814,11 @@
           <t>- Chọn xoá phía tôi, tin nhắn biến mất khỏi khung trò chuyện của người dùng
 - Các thành viên khác vẫn nhìn thấy tin nhắn đó bình thường
 - Người dùng có thể xoá cả tin nhắn của mình lẫn của người khác ở phía mình
-- Tin nhắn đã xoá không quay lại kể cả khi tải lại trang hoặc đăng nhập ở thiết bị khác</t>
+- Tin nhắn đã xoá không quay lại kể cả khi tải lại trang hoặc đăng nhập ở thiết bị khác
+- Thao tác xoá phía tôi nằm trong trình đơn ngữ cảnh của tin nhắn, tách bạch rõ với thu hồi để tránh chọn nhầm
+- Sau khi xoá, các tin nhắn còn lại được nối liền mạch, không để lại khoảng trống
+- Xoá thất bại thì tin nhắn xuất hiện trở lại kèm thông báo lỗi
+- Trình đơn ngữ cảnh của tin nhắn mở được bằng bàn phím và đóng bằng phím Esc</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
@@ -1670,11 +1832,11 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="141" customHeight="1">
-      <c r="A35" s="7" t="n">
+    <row r="35" ht="285" customHeight="1">
+      <c r="A35" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Xử lý lỗi khi gửi tin nhắn</t>
         </is>
@@ -1690,7 +1852,12 @@
 - Thông báo lỗi phân biệt rõ lỗi có thể thử lại và lỗi không thể thử lại như thiếu quyền hoặc dữ liệu sai
 - Bấm gửi lại, hệ thống dùng lại đúng mã tin nhắn ban đầu để không tạo bản trùng
 - Nội dung tin nhắn thất bại được giữ lại cho tới khi gửi thành công hoặc người dùng chủ động xoá
-- Khi phiên đăng nhập không hợp lệ, hệ thống báo lỗi rõ ràng và hướng người dùng đăng nhập lại</t>
+- Khi phiên đăng nhập không hợp lệ, hệ thống báo lỗi rõ ràng và hướng người dùng đăng nhập lại
+- Tin nhắn lỗi hiển thị bằng dấu hiệu trực quan riêng kèm nhãn chữ, không chỉ dựa vào màu
+- Có thao tác xoá tin nhắn lỗi khỏi hàng chờ khi người dùng không muốn gửi lại nữa
+- Nhiều tin nhắn lỗi cùng lúc có thể gửi lại toàn bộ trong một thao tác
+- Tin nhắn chờ gửi vẫn còn sau khi tải lại trang, không biến mất cùng nội dung người dùng đã soạn
+- Khi kết nối trở lại, hệ thống gợi ý gửi lại thay vì tự gửi ngầm khiến người dùng bất ngờ</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
@@ -1704,11 +1871,11 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="111" customHeight="1">
-      <c r="A36" s="7" t="n">
+    <row r="36" ht="225" customHeight="1">
+      <c r="A36" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Chịu tải cao khi nhiều người nhắn cùng lúc</t>
         </is>
@@ -1724,7 +1891,10 @@
 - Khi cơ sở dữ liệu chậm hoặc tạm gián đoạn, tin nhắn không bị mất mà được ghi bổ sung khi hệ thống phục hồi
 - Thứ tự tin nhắn trong một cuộc trò chuyện luôn được giữ đúng theo thời gian gửi
 - Không xảy ra tin nhắn trùng lặp kể cả khi hệ thống xử lý lại một sự kiện
-- Người dùng không nhận thấy sự khác biệt về giao diện giữa lúc tải thấp và tải cao</t>
+- Người dùng không nhận thấy sự khác biệt về giao diện giữa lúc tải thấp và tải cao
+- Giao diện không đứng hình khi nhận nhiều tin nhắn liên tiếp trong thời gian ngắn
+- Khung chat giới hạn số tin nhắn giữ trong bộ nhớ và giải phóng phần ngoài khung nhìn để trình duyệt không phình bộ nhớ
+- Chỉ báo đang gõ và trạng thái đã đọc được gộp cập nhật, không gây dựng lại toàn bộ danh sách tin nhắn</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
@@ -1738,147 +1908,163 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="126" customHeight="1">
-      <c r="A37" s="2" t="n">
+    <row r="37" ht="240" customHeight="1">
+      <c r="A37" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>Hiển thị trạng thái đang gõ</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Là người dùng đang chờ phản hồi, tôi muốn biết đối phương đang gõ tin nhắn, để tôi kiên nhẫn chờ thay vì nghĩ họ đã bỏ đi.</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>- Khi một thành viên bắt đầu gõ, các thành viên khác đang mở cuộc trò chuyện thấy dấu hiệu đang gõ kèm tên người đó
 - Khi người đó ngừng gõ một lúc hoặc gửi tin nhắn, dấu hiệu đang gõ biến mất
 - Trong nhóm có nhiều người cùng gõ, hệ thống hiển thị gộp thay vì liệt kê tràn màn hình
 - Người dùng rời khỏi cuộc trò chuyện hoặc mất kết nối thì dấu hiệu đang gõ của họ được gỡ bỏ tự động
-- Trạng thái đang gõ chỉ gửi tới thành viên của đúng cuộc trò chuyện đó</t>
-        </is>
-      </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
+- Trạng thái đang gõ chỉ gửi tới thành viên của đúng cuộc trò chuyện đó
+- Sự kiện đang gõ được tiết chế tần suất, gõ liên tục không tạo ra luồng sự kiện dày đặc
+- Chỉ báo đang gõ chiếm chỗ cố định trong bố cục, xuất hiện và biến mất không làm nhảy danh sách tin nhắn
+- Chỉ báo tự tắt sau một khoảng nếu không nhận thêm tín hiệu, tránh kẹt vĩnh viễn khi mất kết nối
+- Chỉ báo đang gõ có phần mô tả bằng chữ cho trình đọc màn hình, không chỉ là ba chấm nhấp nháy</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
         <is>
           <t>Tín hiệu đang gõ là dấu hiệu xã hội nhỏ nhưng tạo cảm giác có người thật ở đầu bên kia, làm nhịp hội thoại tự nhiên hơn đáng kể.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="111" customHeight="1">
-      <c r="A38" s="2" t="n">
+    <row r="38" ht="255" customHeight="1">
+      <c r="A38" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>Đánh dấu tin nhắn đã đọc</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>Là người dùng vừa mở một cuộc trò chuyện, tôi muốn các tin nhắn được tự động đánh dấu đã đọc, để tôi không phải thao tác thủ công.</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>- Mở cuộc trò chuyện và cuộn tới tin nhắn mới nhất, hệ thống tự đánh dấu các tin nhắn đó là đã đọc
 - Số tin chưa đọc của cuộc trò chuyện trở về không ngay trên danh sách hội thoại
 - Trạng thái đã đọc được đồng bộ trên tất cả thiết bị mà người dùng đang đăng nhập
 - Tin nhắn chỉ được đánh dấu đã đọc khi người dùng thực sự nhìn thấy, không phải chỉ vì tin nhắn đã tải về
-- Người dùng không thể đánh dấu đã đọc thay cho người khác</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
+- Người dùng không thể đánh dấu đã đọc thay cho người khác
+- Trạng thái đã đọc chỉ được gửi khi cửa sổ trình duyệt đang hiển thị, không gửi khi tab bị ẩn
+- Nhiều tin nhắn cùng đọc trong thời gian ngắn được gộp thành một lần báo lên máy chủ
+- Báo đã đọc thất bại thì được thử lại khi có kết nối, không làm số chưa đọc kẹt sai vĩnh viễn
+- Số chưa đọc trên danh sách hội thoại giảm ngay khi đánh dấu, không chờ máy chủ phản hồi mới cập nhật</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
         <is>
           <t>Đếm tin chưa đọc chính xác là cơ sở để người dùng quyết định vào cuộc trò chuyện nào trước. Đánh dấu sai làm mất niềm tin vào toàn bộ hệ thống chỉ báo.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="111" customHeight="1">
-      <c r="A39" s="2" t="n">
+    <row r="39" ht="225" customHeight="1">
+      <c r="A39" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>Xem ai đã đọc tin nhắn của mình</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>Là người gửi, tôi muốn biết những ai đã đọc tin nhắn của mình, để nắm được thông tin đã tới đích hay chưa.</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>- Tin nhắn cuối cùng đã được đọc hiển thị ảnh đại diện nhỏ của những người đã đọc
 - Trong nhóm, người gửi xem được danh sách đầy đủ những ai đã đọc và ai chưa
 - Trạng thái đã đọc cập nhật tức thời cho người gửi khi người nhận mở cuộc trò chuyện
 - Khi nhiều người cùng đọc trong thời gian ngắn, hệ thống cập nhật gộp thay vì gửi từng thông báo riêng lẻ
-- Chỉ thành viên của cuộc trò chuyện xem được thông tin đã đọc</t>
-        </is>
-      </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
+- Chỉ thành viên của cuộc trò chuyện xem được thông tin đã đọc
+- Ảnh đại diện người đã đọc hiển thị tối đa một số lượng nhất định, phần dư gộp thành chỉ số dạng cộng thêm
+- Danh sách chi tiết ai đã đọc mở được bằng bàn phím và cuộn riêng khi nhóm đông người
+- Mỗi ảnh đại diện có nhãn tên để trình đọc màn hình và người dùng di chuột đều biết đó là ai
+- Trạng thái đã đọc không làm dịch chuyển bố cục tin nhắn khi xuất hiện</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
         <is>
           <t>Biên nhận đã đọc giảm sự mơ hồ trong giao tiếp bất đồng bộ. Việc gộp cập nhật theo lô giữ cho hệ thống không bị quá tải trong nhóm đông người.</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="96" customHeight="1">
-      <c r="A40" s="2" t="n">
+    <row r="40" ht="210" customHeight="1">
+      <c r="A40" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Xem số tin nhắn chưa đọc</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>Là người dùng bận rộn, tôi muốn nhìn thấy số tin nhắn chưa đọc ở từng cuộc trò chuyện, để ưu tiên đọc những gì quan trọng trước.</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>- Mỗi cuộc trò chuyện có tin chưa đọc hiển thị con số chính xác trên danh sách hội thoại
 - Tổng số tin chưa đọc được hiển thị trên biểu tượng ứng dụng hoặc thanh điều hướng
 - Số đếm giảm ngay khi người dùng đọc, không cần tải lại trang
 - Tin nhắn do chính người dùng gửi không bao giờ được tính vào số chưa đọc
-- Số đếm nhất quán giữa các thiết bị của cùng một người dùng</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
+- Số đếm nhất quán giữa các thiết bị của cùng một người dùng
+- Số chưa đọc lớn hơn ngưỡng hiển thị được rút gọn thành dạng có dấu cộng thay vì tràn khỏi huy hiệu
+- Huy hiệu số chưa đọc có nhãn chữ đầy đủ cho trình đọc màn hình
+- Tổng số chưa đọc lấy từ máy chủ, không tính từ số cuộc trò chuyện đã tải về nên vẫn đúng khi danh sách chưa tải hết
+- Số chưa đọc được cập nhật ngay khi có tin nhắn mới đến, kể cả khi người dùng đang ở trang khác</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>Chỉ báo chưa đọc là công cụ ưu tiên công việc hằng ngày. Sai lệch trong con số này khiến người dùng bỏ sót tin quan trọng hoặc mất thời gian kiểm tra thừa.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="126" customHeight="1">
-      <c r="A41" s="7" t="n">
+    <row r="41" ht="285" customHeight="1">
+      <c r="A41" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>Đính kèm ảnh, video và tệp vào tin nhắn</t>
         </is>
@@ -1894,7 +2080,12 @@
 - Trong lúc tải lên, tin nhắn hiển thị tiến độ để người dùng biết còn bao lâu
 - Người dùng gửi được nhiều tệp trong cùng một tin nhắn
 - Tệp được tải trực tiếp lên kho lưu trữ bằng đường dẫn có chữ ký thời hạn, không đi vòng qua máy chủ ứng dụng
-- Tải lên thất bại thì tin nhắn hiển thị lỗi kèm nút thử lại, không tạo tin nhắn rỗng</t>
+- Tải lên thất bại thì tin nhắn hiển thị lỗi kèm nút thử lại, không tạo tin nhắn rỗng
+- Tiến độ tải lên hiển thị theo phần trăm thực tế và có nút huỷ trong lúc đang tải
+- Rời khỏi trang khi còn tệp đang tải lên thì hệ thống cảnh báo trước khi thoát
+- Nhiều tệp trong một tin nhắn được tải lên song song có giới hạn, không mở đồng thời quá nhiều kết nối
+- Tải lên thất bại một tệp trong nhóm thì chỉ tệp đó báo lỗi, các tệp còn lại vẫn giữ nguyên kết quả
+- Khu vực kéo thả có phản hồi trực quan rõ khi tệp được kéo vào và trở lại bình thường khi kéo ra</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
@@ -1908,11 +2099,11 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="96" customHeight="1">
-      <c r="A42" s="7" t="n">
+    <row r="42" ht="240" customHeight="1">
+      <c r="A42" s="8" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>Xem trước tệp trước khi gửi</t>
         </is>
@@ -1928,7 +2119,12 @@
 - Mỗi tệp hiển thị tên và dung lượng để người dùng đối chiếu
 - Người dùng gỡ bỏ được từng tệp khỏi danh sách trước khi gửi
 - Xem trước hoạt động ngay trên trình duyệt, không cần tải tệp lên máy chủ trước
-- Tệp không tạo được ảnh xem trước vẫn hiển thị biểu tượng mặc định thay vì báo lỗi</t>
+- Tệp không tạo được ảnh xem trước vẫn hiển thị biểu tượng mặc định thay vì báo lỗi
+- Ảnh xem trước giữ đúng tỉ lệ, không bị bóp méo với ảnh dọc hay ảnh vuông
+- Ảnh xem trước được giải phóng khỏi bộ nhớ khi tệp bị gỡ hoặc tin nhắn đã gửi xong
+- Dung lượng tệp hiển thị theo đơn vị dễ đọc thay vì số byte thô
+- Vùng xem trước cuộn ngang được khi chọn nhiều tệp và không đẩy ô soạn thảo ra khỏi màn hình
+- Mỗi tệp có nút gỡ riêng thao tác được bằng bàn phím kèm nhãn nêu rõ gỡ tệp nào</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
@@ -1942,11 +2138,11 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="141" customHeight="1">
-      <c r="A43" s="7" t="n">
+    <row r="43" ht="255" customHeight="1">
+      <c r="A43" s="8" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>Giới hạn định dạng và kích thước tệp</t>
         </is>
@@ -1962,7 +2158,11 @@
 - Tệp có định dạng ngoài danh sách bị từ chối ngay khi chọn, kèm thông báo nêu rõ các định dạng được hỗ trợ
 - Tệp vượt quá dung lượng tối đa bị từ chối trước khi bắt đầu tải lên
 - Kiểm tra định dạng được thực hiện ở cả trình duyệt và máy chủ, không tin tưởng hoàn toàn vào phía trình duyệt
-- Đường dẫn tải lên có chữ ký chỉ hợp lệ trong thời gian ngắn và chỉ dùng được cho đúng tệp đã khai báo</t>
+- Đường dẫn tải lên có chữ ký chỉ hợp lệ trong thời gian ngắn và chỉ dùng được cho đúng tệp đã khai báo
+- Thông báo từ chối nêu rõ tên tệp, lý do từ chối và giới hạn cụ thể đang áp dụng
+- Hộp thoại chọn tệp lọc sẵn theo các định dạng được phép để giảm khả năng chọn nhầm
+- Chọn nhiều tệp cùng lúc trong đó có tệp không hợp lệ thì các tệp hợp lệ vẫn được giữ lại
+- Giới hạn dung lượng và danh sách định dạng được nêu sẵn trên giao diện trước khi người dùng chọn tệp</t>
         </is>
       </c>
       <c r="E43" s="11" t="inlineStr">
@@ -1976,11 +2176,11 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="96" customHeight="1">
-      <c r="A44" s="7" t="n">
+    <row r="44" ht="225" customHeight="1">
+      <c r="A44" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>Xem ảnh và video ngay trong khung chat</t>
         </is>
@@ -1996,7 +2196,12 @@
 - Bấm vào ảnh mở chế độ xem toàn màn hình, hỗ trợ chuyển qua lại giữa các ảnh trong cùng cuộc trò chuyện
 - Video có trình phát ngay tại chỗ với nút phát, tạm dừng và thanh thời gian
 - Tài liệu hiển thị tên, dung lượng và nút tải xuống
-- Ảnh và video chỉ tải khi cuộn tới vị trí của chúng để tiết kiệm dữ liệu</t>
+- Ảnh và video chỉ tải khi cuộn tới vị trí của chúng để tiết kiệm dữ liệu
+- Ảnh trong bong bóng tin nhắn có kích thước chỗ dành sẵn nên khung chat không nhảy khi ảnh tải xong
+- Chế độ xem toàn màn hình đóng được bằng phím Esc, chuyển ảnh bằng phím mũi tên và có nút tải xuống
+- Ảnh tải lỗi hiển thị biểu tượng thay thế kèm nút thử lại, không để ô trống
+- Video không tự phát kèm tiếng khi cuộn tới; người dùng chủ động bấm phát
+- Mỗi ảnh có văn bản thay thế mô tả để trình đọc màn hình không bỏ qua nội dung</t>
         </is>
       </c>
       <c r="E44" s="10" t="inlineStr">
@@ -2010,11 +2215,11 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="111" customHeight="1">
-      <c r="A45" s="7" t="n">
+    <row r="45" ht="225" customHeight="1">
+      <c r="A45" s="8" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
         <is>
           <t>Xem kho ảnh, tệp và liên kết của cuộc trò chuyện</t>
         </is>
@@ -2030,7 +2235,11 @@
 - Mỗi mục hiển thị theo thứ tự mới nhất trước và tải thêm khi người dùng cuộn xuống
 - Bấm vào một mục sẽ nhảy tới đúng tin nhắn gốc chứa nội dung đó
 - Nội dung thuộc tin nhắn đã bị thu hồi hoặc đã xoá phía người dùng không xuất hiện trong kho
-- Chỉ thành viên của cuộc trò chuyện truy cập được kho nội dung này</t>
+- Chỉ thành viên của cuộc trò chuyện truy cập được kho nội dung này
+- Mỗi tab trong kho nội dung có phân trang riêng và giữ nguyên vị trí cuộn khi chuyển qua lại
+- Tab đang rỗng hiển thị trạng thái rỗng riêng cho từng loại nội dung
+- Ảnh thu nhỏ được tải theo lô khi cuộn tới, không tải toàn bộ kho ngay khi mở
+- Tải kho nội dung thất bại thì hiển thị lỗi kèm nút thử lại trong đúng tab đó</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
@@ -2044,129 +2253,146 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="126" customHeight="1">
-      <c r="A46" s="2" t="n">
+    <row r="46" ht="240" customHeight="1">
+      <c r="A46" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>Tạo bình chọn trong cuộc trò chuyện</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>Là thành viên nhóm, tôi muốn tạo một bình chọn với nhiều phương án, để cả nhóm ra quyết định nhanh mà không phải đọc hàng chục tin nhắn.</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>- Người dùng nhập câu hỏi và ít nhất hai phương án, chọn cho phép một hay nhiều lựa chọn, rồi tạo bình chọn
 - Bình chọn xuất hiện như một tin nhắn đặc biệt trong dòng trò chuyện cho tất cả thành viên
 - Câu hỏi rỗng hoặc dưới hai phương án thì không tạo được, hệ thống báo lỗi ngay trên biểu mẫu
 - Phương án trùng nhau bị loại bỏ hoặc cảnh báo trước khi tạo
-- Chỉ thành viên của cuộc trò chuyện mới tạo được bình chọn trong đó</t>
-        </is>
-      </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
+- Chỉ thành viên của cuộc trò chuyện mới tạo được bình chọn trong đó
+- Biểu mẫu cho phép thêm và xoá phương án linh hoạt, tự động dồn thứ tự khi xoá phương án ở giữa
+- Ô câu hỏi và từng phương án đều có giới hạn ký tự kèm bộ đếm
+- Trong lúc tạo, nút tạo hiển thị trạng thái đang xử lý và chặn bấm lặp để không tạo hai bình chọn trùng
+- Tạo thất bại thì toàn bộ nội dung đã nhập được giữ nguyên để thử lại
+- Biểu mẫu thao tác được hoàn toàn bằng bàn phím, thêm phương án mới thì tiêu điểm nhảy vào ô vừa thêm</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
         <is>
           <t>Ra quyết định tập thể trong nhóm chat thường rơi vào hỗn loạn. Bình chọn cấu trúc hoá quá trình này và biến kết quả thành dữ liệu rõ ràng thay vì diễn giải chủ quan.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="111" customHeight="1">
-      <c r="A47" s="2" t="n">
+    <row r="47" ht="255" customHeight="1">
+      <c r="A47" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>Bỏ phiếu cho một bình chọn</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>Là thành viên nhóm, tôi muốn chọn phương án mình đồng tình, để đóng góp ý kiến vào quyết định chung.</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>- Người dùng bấm vào phương án, phiếu được ghi nhận và giao diện phản ánh lựa chọn ngay
 - Với bình chọn một lựa chọn, chọn phương án mới sẽ thay thế phương án cũ
 - Với bình chọn nhiều lựa chọn, người dùng chọn và bỏ chọn được nhiều phương án
 - Bình chọn đã đóng không nhận thêm phiếu, giao diện chuyển sang chế độ chỉ xem
-- Mỗi người chỉ được tính một lượt bỏ phiếu trên mỗi phương án, thao tác lặp không làm sai lệch kết quả</t>
-        </is>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
+- Mỗi người chỉ được tính một lượt bỏ phiếu trên mỗi phương án, thao tác lặp không làm sai lệch kết quả
+- Phương án đang được chọn có dấu hiệu rõ bằng cả hình dạng và chữ, không chỉ bằng màu
+- Giao diện cập nhật lạc quan ngay khi bấm và hoàn nguyên đúng trạng thái cũ nếu máy chủ báo lỗi
+- Bấm liên tiếp vào cùng một phương án không tạo ra nhiều phiếu và không làm số phiếu nhảy loạn
+- Phương án bỏ phiếu được bằng bàn phím và trạng thái chọn được thông báo cho trình đọc màn hình</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
         <is>
           <t>Cơ chế bỏ phiếu phải trực quan và không cho phép gian lận đơn giản, nếu không kết quả sẽ mất giá trị tham khảo trong mắt nhóm.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="96" customHeight="1">
-      <c r="A48" s="2" t="n">
+    <row r="48" ht="240" customHeight="1">
+      <c r="A48" s="4" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>Xem kết quả bình chọn cập nhật tức thời</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>Là thành viên nhóm, tôi muốn thấy kết quả bình chọn thay đổi ngay khi có người bỏ phiếu, để nắm được xu hướng của cả nhóm.</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D48" s="5" t="inlineStr">
         <is>
           <t>- Khi bất kỳ ai bỏ phiếu, số phiếu và tỷ lệ phần trăm của các phương án cập nhật ngay cho mọi người đang mở cuộc trò chuyện
 - Người dùng xem được danh sách những ai đã chọn từng phương án
 - Tổng số người đã tham gia bình chọn được hiển thị rõ
 - Người chưa bỏ phiếu vẫn xem được kết quả hiện tại mà không bị buộc phải chọn trước
-- Cập nhật kết quả chỉ gửi tới thành viên của đúng cuộc trò chuyện chứa bình chọn</t>
-        </is>
-      </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
+- Cập nhật kết quả chỉ gửi tới thành viên của đúng cuộc trò chuyện chứa bình chọn
+- Thanh tỉ lệ phần trăm có chuyển động mượt khi số phiếu thay đổi và tôn trọng thiết lập giảm chuyển động của hệ thống
+- Danh sách người đã chọn từng phương án hiển thị rút gọn kèm lối mở rộng khi đông người
+- Cập nhật kết quả đến liên tục được gộp lại, không dựng lại toàn bộ khối bình chọn mỗi lần có phiếu
+- Tỉ lệ phần trăm làm tròn nhất quán và tổng luôn hợp lý, không hiển thị con số gây hiểu nhầm</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
         <is>
           <t>Kết quả cập nhật trực tiếp tạo động lực tham gia và giúp nhóm nhận ra sớm khi đã đạt được đồng thuận, rút ngắn thời gian ra quyết định.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="96" customHeight="1">
-      <c r="A49" s="2" t="n">
+    <row r="49" ht="180" customHeight="1">
+      <c r="A49" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Đóng bình chọn</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Là người tạo bình chọn, tôi muốn đóng bình chọn khi đã đủ ý kiến, để chốt kết quả và tránh phiếu muộn làm thay đổi quyết định.</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>- Người tạo bấm đóng, bình chọn chuyển sang trạng thái đã đóng cho tất cả thành viên ngay lập tức
 - Sau khi đóng, không ai bỏ thêm phiếu hay thay đổi phiếu đã bỏ được
 - Kết quả cuối cùng vẫn hiển thị đầy đủ trong lịch sử trò chuyện
 - Chỉ người tạo bình chọn hoặc quản trị viên nhóm mới có quyền đóng
-- Bình chọn đã đóng không thể mở lại</t>
+- Bình chọn đã đóng không thể mở lại
+- Thao tác đóng bình chọn hỏi xác nhận và nêu rõ là không mở lại được
+- Sau khi đóng, mọi nút bỏ phiếu chuyển sang trạng thái vô hiệu kèm nhãn đã đóng thay vì biến mất
+- Đóng thất bại thì bình chọn giữ nguyên trạng thái mở kèm thông báo lỗi
+- Nút đóng chỉ hiển thị với người có quyền, không hiện rồi mới báo lỗi khi bấm</t>
         </is>
       </c>
       <c r="E49" s="12" t="inlineStr">
@@ -2174,17 +2400,17 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr">
         <is>
           <t>Chốt thời điểm kết thúc giúp kết quả bình chọn có tính ràng buộc, tránh tranh cãi về việc phiếu nào được tính khi nhóm đã hành động theo kết quả.</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="96" customHeight="1">
-      <c r="A50" s="7" t="n">
+    <row r="50" ht="180" customHeight="1">
+      <c r="A50" s="8" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Xem trạng thái trực tuyến của bạn bè</t>
         </is>
@@ -2199,7 +2425,10 @@
           <t>- Bạn bè đang trực tuyến hiển thị chấm xanh trên ảnh đại diện tại danh sách bạn bè và danh sách hội thoại
 - Trạng thái trực tuyến nhất quán trên mọi màn hình hiển thị người dùng đó
 - Trạng thái được xác định ở mức tài khoản, không phụ thuộc vào một kết nối cụ thể nào
-- Người dùng chỉ xem được trạng thái của bạn bè, không xem được của người lạ</t>
+- Người dùng chỉ xem được trạng thái của bạn bè, không xem được của người lạ
+- Chấm trạng thái có nhãn chữ kèm theo để người dùng không phân biệt được màu vẫn hiểu
+- Trạng thái đang tải hiển thị bằng chấm trung tính thay vì mặc định coi là ngoại tuyến
+- Trạng thái hiển thị nhất quán giữa danh sách bạn bè, danh sách hội thoại và tiêu đề khung chat</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -2213,11 +2442,11 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="96" customHeight="1">
-      <c r="A51" s="7" t="n">
+    <row r="51" ht="180" customHeight="1">
+      <c r="A51" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B51" s="9" t="inlineStr">
         <is>
           <t>Cập nhật trạng thái trực tuyến tức thời</t>
         </is>
@@ -2232,7 +2461,10 @@
           <t>- Khi một người bạn đăng nhập, chấm trạng thái của họ chuyển sang trực tuyến cho tất cả bạn bè đang mở ứng dụng
 - Khi họ đóng ứng dụng hoặc mất mạng, trạng thái chuyển sang ngoại tuyến trong khoảng thời gian ngắn
 - Người dùng không cần tải lại trang để thấy trạng thái mới
-- Thay đổi trạng thái chỉ được thông báo tới bạn bè của người đó</t>
+- Thay đổi trạng thái chỉ được thông báo tới bạn bè của người đó
+- Trạng thái đổi liên tục trong thời gian ngắn được làm mượt, tránh chấm trạng thái nhấp nháy
+- Cập nhật trạng thái không làm sắp xếp lại danh sách đột ngột khi người dùng đang thao tác
+- Sau khi kết nối lại, ứng dụng đồng bộ lại toàn bộ trạng thái thay vì giữ giá trị cũ đã sai</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
@@ -2246,11 +2478,11 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="111" customHeight="1">
-      <c r="A52" s="7" t="n">
+    <row r="52" ht="195" customHeight="1">
+      <c r="A52" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="B52" s="8" t="inlineStr">
+      <c r="B52" s="9" t="inlineStr">
         <is>
           <t>Xem thời điểm hoạt động gần nhất</t>
         </is>
@@ -2265,7 +2497,10 @@
           <t>- Với bạn bè đang ngoại tuyến, hệ thống hiển thị mốc thời gian hoạt động gần nhất theo dạng dễ đọc như "5 phút trước"
 - Mốc thời gian được ghi lại tại thời điểm người dùng ngắt kết nối và được lưu trong khoảng thời gian hợp lý
 - Nếu không có dữ liệu hoạt động gần nhất, hệ thống chỉ hiển thị trạng thái ngoại tuyến, không hiển thị mốc sai
-- Chỉ bạn bè mới xem được thông tin hoạt động gần nhất của nhau</t>
+- Chỉ bạn bè mới xem được thông tin hoạt động gần nhất của nhau
+- Mốc thời gian tương đối tự cập nhật theo thời gian mà không cần tải lại trang
+- Di chuột hoặc chạm giữ vào mốc thời gian hiển thị thời điểm đầy đủ chính xác
+- Mốc thời gian hiển thị bằng tiếng Việt đúng ngữ pháp cho mọi khoảng cách thời gian</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
@@ -2279,11 +2514,11 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="96" customHeight="1">
-      <c r="A53" s="7" t="n">
+    <row r="53" ht="180" customHeight="1">
+      <c r="A53" s="8" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="8" t="inlineStr">
+      <c r="B53" s="9" t="inlineStr">
         <is>
           <t>Giữ trạng thái chính xác khi dùng nhiều thiết bị</t>
         </is>
@@ -2298,7 +2533,9 @@
           <t>- Người dùng chỉ chuyển sang ngoại tuyến khi toàn bộ thiết bị của họ đã ngắt kết nối
 - Đóng một tab hoặc một thiết bị không làm trạng thái chuyển sang ngoại tuyến nếu thiết bị khác còn kết nối
 - Hệ thống định kỳ kiểm tra các kết nối còn sống và tự dọn những kết nối đã chết do mất mạng đột ngột
-- Kết nối bị treo không làm người dùng bị kẹt vĩnh viễn ở trạng thái trực tuyến</t>
+- Kết nối bị treo không làm người dùng bị kẹt vĩnh viễn ở trạng thái trực tuyến
+- Đóng tab đột ngột không làm trạng thái sai quá một khoảng thời gian ngắn xác định
+- Số thiết bị đang kết nối không rò rỉ ra ngoài, người khác chỉ thấy trực tuyến hay không</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
@@ -2312,196 +2549,214 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="111" customHeight="1">
-      <c r="A54" s="2" t="n">
+    <row r="54" ht="225" customHeight="1">
+      <c r="A54" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Bắt đầu cuộc gọi thoại</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn gọi thoại trực tiếp cho một người bạn từ trong cuộc trò chuyện, để trao đổi nhanh những việc khó diễn đạt bằng chữ.</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>- Bấm biểu tượng gọi trong cuộc trò chuyện riêng, hệ thống xin quyền micro và chuyển sang màn hình đang gọi
 - Người nhận thấy màn hình cuộc gọi đến ngay nếu đang trực tuyến
 - Nếu người dùng từ chối cấp quyền micro, hệ thống thông báo rõ lý do và không bắt đầu cuộc gọi
 - Không thể gọi cho người chưa phải bạn bè hoặc trong cuộc trò chuyện nhóm
-- Người gọi có thể huỷ trước khi đối phương bắt máy</t>
-        </is>
-      </c>
-      <c r="E54" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
+- Người gọi có thể huỷ trước khi đối phương bắt máy
+- Nút gọi bị vô hiệu kèm giải thích khi đối phương ngoại tuyến hoặc trong cuộc trò chuyện nhóm
+- Trạng thái xin quyền micro hiển thị rõ ràng, người dùng biết trình duyệt đang chờ mình cho phép
+- Từ chối quyền micro thì hệ thống hướng dẫn cách bật lại quyền trong trình duyệt
+- Màn hình gọi hiển thị đúng tên và ảnh đại diện người được gọi ngay từ lúc bắt đầu</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
         <is>
           <t>Gọi thoại xử lý được những trao đổi mà nhắn tin quá chậm hoặc dễ hiểu nhầm. Đặt nút gọi ngay trong cuộc trò chuyện giữ hành trình người dùng liền mạch.</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="96" customHeight="1">
-      <c r="A55" s="2" t="n">
+    <row r="55" ht="255" customHeight="1">
+      <c r="A55" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Nhận cuộc gọi đến kèm chuông</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Là người nhận, tôi muốn thấy màn hình cuộc gọi đến kèm chuông báo, để không bỏ lỡ cuộc gọi khi đang làm việc khác.</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>- Màn hình cuộc gọi đến hiển thị tên và ảnh đại diện của người gọi kèm hai nút chấp nhận và từ chối
 - Chuông báo phát cho tới khi người dùng phản hồi hoặc cuộc gọi kết thúc
 - Màn hình cuộc gọi đến hiện ra dù người dùng đang ở bất kỳ trang nào trong ứng dụng
 - Chuông dừng ngay khi cuộc gọi được chấp nhận, bị từ chối hoặc người gọi huỷ
-- Nếu người dùng đang trong một cuộc gọi khác, cuộc gọi mới được xử lý là máy bận</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
+- Nếu người dùng đang trong một cuộc gọi khác, cuộc gọi mới được xử lý là máy bận
+- Chuông tôn trọng thiết lập âm thanh của ứng dụng và có nút tắt tiếng nhanh ngay trên màn hình cuộc gọi đến
+- Màn hình cuộc gọi đến hiển thị trên mọi trang mà không làm mất thao tác đang dở phía dưới
+- Trình duyệt chặn tự phát âm thanh thì hệ thống vẫn hiển thị cuộc gọi đến bằng hình ảnh rõ ràng
+- Hai nút chấp nhận và từ chối đủ lớn, cách xa nhau để tránh bấm nhầm và thao tác được bằng bàn phím</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>Cuộc gọi là hình thức giao tiếp đồng bộ, chỉ có giá trị nếu người nhận biết ngay. Hiển thị ở cấp toàn ứng dụng đảm bảo không bỏ lỡ dù đang ở màn hình nào.</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="111" customHeight="1">
-      <c r="A56" s="2" t="n">
+    <row r="56" ht="210" customHeight="1">
+      <c r="A56" s="4" t="n">
         <v>55</v>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>Chấp nhận cuộc gọi</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Là người nhận, tôi muốn bấm chấp nhận để bắt đầu nói chuyện, để kết nối thoại được thiết lập nhanh và ổn định.</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>- Bấm chấp nhận, hệ thống xin quyền micro và thiết lập kết nối thoại với người gọi
 - Cả hai bên chuyển sang màn hình đang trong cuộc gọi kèm đồng hồ đếm thời gian
 - Âm thanh được truyền trực tiếp giữa hai máy, máy chủ chỉ làm nhiệm vụ kết nối ban đầu
 - Người dùng bật tắt micro được trong lúc gọi
-- Nếu không thiết lập được kết nối, hệ thống thông báo lỗi và kết thúc cuộc gọi thay vì treo vô hạn</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
+- Nếu không thiết lập được kết nối, hệ thống thông báo lỗi và kết thúc cuộc gọi thay vì treo vô hạn
+- Màn hình trong cuộc gọi hiển thị trạng thái kết nối theo từng giai đoạn thay vì chỉ một màn hình tĩnh
+- Nút tắt micro phản ánh đúng trạng thái hiện tại bằng cả biểu tượng và chữ
+- Chất lượng kết nối kém được báo cho người dùng thay vì để họ tự đoán vì sao nghe ngắt quãng</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
         <is>
           <t>Truyền âm thanh trực tiếp giữa hai máy giảm độ trễ và loại bỏ chi phí băng thông cho máy chủ, cho phép mở rộng tính năng gọi mà chi phí hạ tầng gần như không tăng.</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="81" customHeight="1">
-      <c r="A57" s="2" t="n">
+    <row r="57" ht="135" customHeight="1">
+      <c r="A57" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>Từ chối cuộc gọi</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Là người nhận đang bận, tôi muốn từ chối cuộc gọi, để người gọi biết ngay và không phải chờ.</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>- Bấm từ chối, chuông tắt và màn hình cuộc gọi đến đóng lại ngay
 - Người gọi nhận thông báo cuộc gọi bị từ chối và màn hình gọi của họ cũng đóng
 - Không có kết nối âm thanh nào được thiết lập, quyền micro không bị yêu cầu
-- Cuộc gọi bị từ chối được ghi nhận trong cuộc trò chuyện dưới dạng tin nhắn hệ thống</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
+- Cuộc gọi bị từ chối được ghi nhận trong cuộc trò chuyện dưới dạng tin nhắn hệ thống
+- Nút từ chối phản hồi tức thì trên giao diện, không chờ máy chủ xác nhận mới đóng màn hình
+- Từ chối rồi thì màn hình cuộc gọi đến không bật lại do sự kiện đến trễ</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>Từ chối rõ ràng tôn trọng thời gian của cả hai phía và tránh việc người gọi hiểu nhầm là mất kết nối kỹ thuật.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="96" customHeight="1">
-      <c r="A58" s="2" t="n">
+    <row r="58" ht="195" customHeight="1">
+      <c r="A58" s="4" t="n">
         <v>57</v>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr">
         <is>
           <t>Kết thúc cuộc gọi</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>Là người tham gia cuộc gọi, tôi muốn kết thúc cuộc gọi bất cứ lúc nào, để chủ động khép lại khi đã trao đổi xong.</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>- Bên nào bấm kết thúc thì cả hai phía đều thoát khỏi màn hình cuộc gọi ngay lập tức
 - Micro được giải phóng, đèn báo sử dụng micro của trình duyệt tắt hoàn toàn
 - Thời lượng cuộc gọi được ghi lại trong cuộc trò chuyện dưới dạng tin nhắn hệ thống
 - Nếu một bên mất mạng đột ngột, bên còn lại vẫn được đưa về trạng thái kết thúc thay vì kẹt ở màn hình gọi
-- Sau khi kết thúc, hai bên có thể gọi lại ngay mà không cần tải lại trang</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
+- Sau khi kết thúc, hai bên có thể gọi lại ngay mà không cần tải lại trang
+- Sau khi kết thúc, giao diện trở lại đúng cuộc trò chuyện trước đó chứ không về màn hình mặc định
+- Mọi tài nguyên âm thanh và kết nối được giải phóng, kiểm chứng được bằng việc đèn micro của trình duyệt tắt
+- Bấm kết thúc nhiều lần không gây lỗi hoặc gửi nhiều lần sự kiện kết thúc</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
         <is>
           <t>Giải phóng tài nguyên micro triệt để là yêu cầu bắt buộc về quyền riêng tư. Kẹt ở màn hình gọi khi mất mạng là lỗi nghiêm trọng về trải nghiệm cần được xử lý chủ động.</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="126" customHeight="1">
-      <c r="A59" s="2" t="n">
+    <row r="59" ht="210" customHeight="1">
+      <c r="A59" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>Thiết lập kết nối thoại ổn định</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Là người dùng ở các điều kiện mạng khác nhau, tôi muốn cuộc gọi vẫn kết nối được, để tính năng dùng được ngoài môi trường mạng lý tưởng.</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>- Hai máy tự động trao đổi thông tin đường mạng để tìm ra tuyến kết nối tốt nhất
 - Cuộc gọi vẫn thiết lập được khi hai bên ở sau bộ định tuyến gia đình khác nhau
 - Trong lúc dò tìm tuyến kết nối, người dùng thấy trạng thái đang kết nối thay vì màn hình đứng im
 - Nếu sau một khoảng thời gian vẫn không kết nối được, hệ thống thông báo thất bại và kết thúc cuộc gọi
-- Thông tin trao đổi để thiết lập kết nối chỉ được chuyển tới đúng hai người trong cuộc gọi</t>
+- Thông tin trao đổi để thiết lập kết nối chỉ được chuyển tới đúng hai người trong cuộc gọi
+- Trong lúc dò tuyến kết nối, giao diện hiển thị tiến trình theo từng bước để người dùng biết hệ thống đang làm gì
+- Thời gian chờ tối đa được nêu rõ và có nút huỷ chủ động thay vì bắt người dùng chờ hết giờ</t>
         </is>
       </c>
       <c r="E59" s="12" t="inlineStr">
@@ -2509,51 +2764,54 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="F59" s="5" t="inlineStr">
         <is>
           <t>Phần lớn người dùng nằm sau các lớp mạng nội bộ. Quá trình dò tìm tuyến kết nối là điều kiện kỹ thuật bắt buộc để gọi trực tiếp giữa hai máy hoạt động được trong thực tế.</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="126" customHeight="1">
-      <c r="A60" s="2" t="n">
+    <row r="60" ht="210" customHeight="1">
+      <c r="A60" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>Xử lý cuộc gọi không được trả lời</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Là người gọi, tôi muốn hệ thống tự kết thúc khi đối phương không bắt máy, để tôi không phải chờ vô thời hạn.</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>- Sau một khoảng thời gian đổ chuông mà không có phản hồi, hệ thống tự kết thúc cuộc gọi ở cả hai phía
 - Người gọi nhận thông báo cuộc gọi nhỡ, người nhận thấy ghi nhận cuộc gọi nhỡ trong cuộc trò chuyện
 - Gọi cho người đang ngoại tuyến, hệ thống báo ngay là không thể kết nối thay vì đổ chuông vô ích
 - Chuông báo phía người nhận tự tắt khi hết thời gian chờ
-- Cuộc gọi nhỡ được ghi lại dưới dạng tin nhắn hệ thống trong cuộc trò chuyện</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
+- Cuộc gọi nhỡ được ghi lại dưới dạng tin nhắn hệ thống trong cuộc trò chuyện
+- Thời gian đổ chuông còn lại hiển thị được cho người gọi thay vì chờ trong vô định
+- Tin nhắn hệ thống ghi nhận cuộc gọi nhỡ có nút gọi lại ngay tại chỗ
+- Cuộc gọi nhỡ được tính vào số chưa đọc của cuộc trò chuyện như một sự kiện cần chú ý</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
         <is>
           <t>Giới hạn thời gian đổ chuông và ghi nhận cuộc gọi nhỡ giúp cả hai phía không rơi vào trạng thái treo, đồng thời để lại dấu vết để liên hệ lại sau.</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="126" customHeight="1">
-      <c r="A61" s="7" t="n">
+    <row r="61" ht="225" customHeight="1">
+      <c r="A61" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="8" t="inlineStr">
+      <c r="B61" s="9" t="inlineStr">
         <is>
           <t>Nhận thông báo tức thời trong ứng dụng</t>
         </is>
@@ -2569,7 +2827,10 @@
 - Bấm vào thông báo sẽ mở đúng nội dung liên quan, ví dụ đúng cuộc trò chuyện hoặc đúng lời mời
 - Thông báo chỉ được gửi tới đúng người dùng liên quan, không rò rỉ sang tài khoản khác
 - Người dùng đang ngoại tuyến vẫn thấy đầy đủ thông báo khi mở lại ứng dụng
-- Người dùng đã tắt kênh thông báo trong ứng dụng thì không nhận thông báo loại đó</t>
+- Người dùng đã tắt kênh thông báo trong ứng dụng thì không nhận thông báo loại đó
+- Thông báo mới xuất hiện có chuyển động vào nhẹ nhàng và tôn trọng thiết lập giảm chuyển động của hệ thống
+- Nhiều thông báo đến dồn dập được gộp hiển thị thay vì đẩy một chuỗi dài che màn hình
+- Thông báo có nội dung dài được cắt gọn với số dòng cố định, xem đầy đủ khi mở chi tiết</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
@@ -2583,11 +2844,11 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="81" customHeight="1">
-      <c r="A62" s="7" t="n">
+    <row r="62" ht="225" customHeight="1">
+      <c r="A62" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="B62" s="8" t="inlineStr">
+      <c r="B62" s="9" t="inlineStr">
         <is>
           <t>Xem danh sách thông báo</t>
         </is>
@@ -2603,7 +2864,12 @@
 - Thông báo chưa đọc được đánh dấu khác biệt rõ ràng so với thông báo đã đọc
 - Danh sách tải thêm khi người dùng cuộn xuống thay vì tải toàn bộ một lần
 - Mỗi thông báo hiển thị nội dung, loại sự kiện và thời điểm xảy ra
-- Người dùng chỉ xem được thông báo của chính mình</t>
+- Người dùng chỉ xem được thông báo của chính mình
+- Bảng thông báo tải thêm theo trang khi cuộn và không gọi trùng cùng một trang khi cuộn nhanh
+- Phân trang không lặp lại hay bỏ sót mục khi có thông báo mới đến giữa lúc đang tải thêm
+- Đã tải hết danh sách thì hiển thị dòng báo đã xem hết thay vì im lặng ngừng tải
+- Trang đầu hiển thị khung xương trong lúc tải; tải thất bại thì hiển thị lỗi kèm nút thử lại ngay trong bảng
+- Bảng thông báo mở và đóng được bằng bàn phím, danh sách di chuyển được bằng phím mũi tên</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
@@ -2617,11 +2883,11 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="81" customHeight="1">
-      <c r="A63" s="7" t="n">
+    <row r="63" ht="165" customHeight="1">
+      <c r="A63" s="8" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="8" t="inlineStr">
+      <c r="B63" s="9" t="inlineStr">
         <is>
           <t>Đánh dấu thông báo đã đọc</t>
         </is>
@@ -2637,7 +2903,10 @@
 - Nút đánh dấu tất cả đã đọc xoá toàn bộ trạng thái chưa đọc trong một thao tác
 - Số đếm chưa đọc cập nhật ngay sau mỗi thao tác, không cần tải lại trang
 - Thao tác chỉ ảnh hưởng tới thông báo của chính người dùng
-- Thông báo đã đọc vẫn nằm trong danh sách để tra cứu lại sau</t>
+- Thông báo đã đọc vẫn nằm trong danh sách để tra cứu lại sau
+- Đánh dấu đã đọc cập nhật giao diện ngay lập tức và hoàn nguyên nếu máy chủ báo lỗi
+- Nút đánh dấu tất cả đã đọc hiển thị trạng thái đang xử lý và bị vô hiệu khi không còn mục chưa đọc
+- Thao tác đánh dấu không làm danh sách nhảy vị trí hay đóng bảng thông báo</t>
         </is>
       </c>
       <c r="E63" s="10" t="inlineStr">
@@ -2651,11 +2920,11 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="81" customHeight="1">
-      <c r="A64" s="7" t="n">
+    <row r="64" ht="150" customHeight="1">
+      <c r="A64" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="B64" s="8" t="inlineStr">
+      <c r="B64" s="9" t="inlineStr">
         <is>
           <t>Xem số thông báo chưa đọc</t>
         </is>
@@ -2670,7 +2939,10 @@
           <t>- Biểu tượng chuông hiển thị con số chính xác các thông báo chưa đọc
 - Số đếm tăng ngay khi có thông báo mới và giảm ngay khi người dùng đọc
 - Khi không còn thông báo chưa đọc, con số biến mất hoàn toàn thay vì hiển thị số không
-- Số đếm đồng bộ giữa các thiết bị của cùng một người dùng</t>
+- Số đếm đồng bộ giữa các thiết bị của cùng một người dùng
+- Số chưa đọc trên chuông lấy từ máy chủ chứ không đếm từ danh sách đã tải, nên vẫn đúng khi có nhiều hơn một trang
+- Số vượt ngưỡng hiển thị được rút gọn nhưng nhãn cho trình đọc màn hình vẫn nêu con số đầy đủ
+- Số đếm được đồng bộ lại sau khi kết nối thời gian thực khôi phục</t>
         </is>
       </c>
       <c r="E64" s="10" t="inlineStr">
@@ -2684,11 +2956,11 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="96" customHeight="1">
-      <c r="A65" s="7" t="n">
+    <row r="65" ht="270" customHeight="1">
+      <c r="A65" s="8" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="8" t="inlineStr">
+      <c r="B65" s="9" t="inlineStr">
         <is>
           <t>Tuỳ chỉnh kênh nhận thông báo</t>
         </is>
@@ -2704,7 +2976,12 @@
 - Người dùng đặt riêng cấu hình cho từng loại sự kiện, ghi đè lên cấu hình chung
 - Có công tắc tổng để tắt toàn bộ thông báo trong một thao tác
 - Cấu hình có hiệu lực ngay lập tức, sự kiện sinh ra sau đó tuân theo cấu hình mới
-- Người dùng chưa từng cấu hình thì áp dụng giá trị mặc định bật tất cả các kênh</t>
+- Người dùng chưa từng cấu hình thì áp dụng giá trị mặc định bật tất cả các kênh
+- Mỗi công tắc phản hồi ngay khi bật tắt và tự hoàn nguyên nếu lưu thất bại, kèm thông báo lỗi
+- Công tắc tổng khi tắt sẽ làm mờ và vô hiệu các công tắc con để người dùng hiểu vì sao chúng không còn tác dụng
+- Trang cấu hình hiển thị khung xương trong lúc tải và có nút thử lại khi tải thất bại
+- Mọi công tắc thao tác được bằng bàn phím và có nhãn mô tả rõ ràng, không chỉ dựa vào vị trí trong bảng
+- Trang có nút khôi phục về giá trị mặc định</t>
         </is>
       </c>
       <c r="E65" s="10" t="inlineStr">
@@ -2718,11 +2995,11 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="126" customHeight="1">
-      <c r="A66" s="7" t="n">
+    <row r="66" ht="225" customHeight="1">
+      <c r="A66" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="B66" s="8" t="inlineStr">
+      <c r="B66" s="9" t="inlineStr">
         <is>
           <t>Nhận email tổng hợp khi có nhiều thông báo chưa đọc</t>
         </is>
@@ -2738,7 +3015,10 @@
 - Giữa hai lần gửi luôn có khoảng nghỉ tối thiểu để tránh gửi liên tục
 - Người dùng đã tắt kênh email hoặc tắt tính năng tổng hợp thì không nhận email này
 - Email tổng hợp không bao gồm nội dung chi tiết tin nhắn riêng tư, chỉ nêu số lượng và loại sự kiện
-- Người dùng đang trực tuyến vẫn nhận được thông báo tổng hợp trong ứng dụng tương ứng</t>
+- Người dùng đang trực tuyến vẫn nhận được thông báo tổng hợp trong ứng dụng tương ứng
+- Email tổng hợp hiển thị đúng trên các ứng dụng thư phổ biến và có cả bản văn bản thuần cho ứng dụng không hiển thị HTML
+- Email có liên kết dẫn thẳng tới trang cấu hình thông báo để người dùng tắt nếu không muốn nhận
+- Tiêu đề email nêu rõ số lượng sự kiện chưa đọc để người dùng quyết định mở hay không</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
@@ -2752,129 +3032,141 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="141" customHeight="1">
-      <c r="A67" s="2" t="n">
+    <row r="67" ht="255" customHeight="1">
+      <c r="A67" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="5" t="inlineStr">
         <is>
           <t>Xem danh sách gợi ý kết bạn</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C67" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn xem những người hệ thống gợi ý, để mở rộng mạng lưới mà không phải tự tìm kiếm thủ công.</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>- Hệ thống hiển thị danh sách người dùng được gợi ý kèm ảnh đại diện, giới thiệu ngắn và lý do gợi ý
 - Người đã là bạn bè hoặc đã có lời mời đang chờ không xuất hiện trong danh sách gợi ý
 - Người dùng gửi được lời mời kết bạn ngay từ thẻ gợi ý và thẻ đó biến mất khỏi danh sách
 - Danh sách được tính sẵn và làm mới định kỳ để mở nhanh, không bắt người dùng chờ tính toán
-- Chính người dùng không bao giờ xuất hiện trong danh sách gợi ý của mình</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
+- Chính người dùng không bao giờ xuất hiện trong danh sách gợi ý của mình
+- Danh sách gợi ý hiển thị khung xương trong lúc tải và trạng thái rỗng có hướng dẫn khi không có ứng viên
+- Lý do gợi ý được diễn đạt bằng ngôn ngữ đời thường, không hiển thị điểm số kỹ thuật thô
+- Gửi lời mời từ thẻ gợi ý hiển thị trạng thái đang xử lý và hoàn nguyên thẻ nếu thất bại
+- Danh sách tải thêm khi cuộn thay vì giới hạn cứng ở nhóm đầu tiên
+- Có nút làm mới danh sách gợi ý kèm thời điểm cập nhật gần nhất</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
         <is>
           <t>Mạng lưới càng lớn thì giá trị của nền tảng càng cao. Gợi ý chủ động giải quyết vấn đề người dùng không biết bắt đầu tìm ai, đặc biệt với tài khoản mới.</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="96" customHeight="1">
-      <c r="A68" s="2" t="n">
+    <row r="68" ht="210" customHeight="1">
+      <c r="A68" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>Cải thiện gợi ý bằng thẻ sở thích</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn cập nhật các chủ đề mình quan tâm, để hệ thống gợi ý những người có điểm chung với tôi.</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>- Người dùng xem và chỉnh sửa được danh sách thẻ sở thích của mình bất kỳ lúc nào trong phần hồ sơ
 - Sau khi thay đổi sở thích, danh sách gợi ý được tính lại ở lần làm mới kế tiếp
 - Thẻ sở thích chung giữa hai người được hiển thị làm lý do gợi ý
 - Danh sách thẻ chỉ hiển thị các chủ đề đang được kích hoạt bởi hệ thống
-- Người dùng không chọn sở thích nào vẫn nhận được gợi ý dựa trên các tín hiệu khác</t>
-        </is>
-      </c>
-      <c r="E68" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
+- Người dùng không chọn sở thích nào vẫn nhận được gợi ý dựa trên các tín hiệu khác
+- Thay đổi sở thích được lưu với phản hồi rõ ràng và có thể huỷ bỏ thay đổi chưa lưu
+- Thẻ sở thích chung được làm nổi bật trong thẻ gợi ý để người dùng thấy ngay điểm chung
+- Danh sách thẻ dài có ô tìm kiếm và nhóm theo chủ đề thay vì một danh sách phẳng khó tìm</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
         <is>
           <t>Sở thích là tín hiệu do chính người dùng khai báo, chất lượng cao và dễ giải thích. Hiển thị điểm chung làm lý do gợi ý giúp người dùng tin tưởng và chấp nhận đề xuất.</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="126" customHeight="1">
-      <c r="A69" s="2" t="n">
+    <row r="69" ht="180" customHeight="1">
+      <c r="A69" s="4" t="n">
         <v>68</v>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" s="5" t="inlineStr">
         <is>
           <t>Nhận gợi ý ngay khi mới tham gia</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C69" s="5" t="inlineStr">
         <is>
           <t>Là người dùng mới chưa có bạn bè nào, tôi muốn vẫn nhận được gợi ý hợp lý, để không rơi vào màn hình trống ngay lần đầu sử dụng.</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>- Khi chưa có dữ liệu quan hệ, hệ thống gợi ý dựa trên sở thích đã khai báo, mức tương đồng phần giới thiệu bản thân và vị trí
 - Danh sách gợi ý được tạo ngay trong lần truy cập đầu tiên, không chờ tới chu kỳ tính toán định kỳ
 - Kết quả gợi ý được lưu lại và có thời hạn để lần mở sau hiển thị tức thì
 - Người dùng vừa kết bạn xong được loại khỏi danh sách gợi ý ngay lập tức
-- Khi không tìm được ứng viên phù hợp, hệ thống hiển thị hướng dẫn tìm kiếm thủ công thay vì màn hình trống</t>
-        </is>
-      </c>
-      <c r="E69" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
+- Khi không tìm được ứng viên phù hợp, hệ thống hiển thị hướng dẫn tìm kiếm thủ công thay vì màn hình trống
+- Trong lần tính gợi ý đầu tiên, giao diện hiển thị trạng thái đang chuẩn bị gợi ý thay vì trạng thái rỗng gây hiểu nhầm
+- Nếu quá trình tính vượt thời gian chờ, hệ thống hiển thị hướng dẫn tìm kiếm thủ công kèm nút thử lại</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
         <is>
           <t>Trải nghiệm những phút đầu tiên quyết định người dùng có quay lại hay không. Xử lý tốt bài toán khởi đầu nguội là yếu tố then chốt giữ chân người dùng mới.</t>
         </is>
       </c>
     </row>
-    <row r="70" ht="141" customHeight="1">
-      <c r="A70" s="2" t="n">
+    <row r="70" ht="195" customHeight="1">
+      <c r="A70" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B70" s="5" t="inlineStr">
         <is>
           <t>Huấn luyện và đánh giá mô hình gợi ý</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C70" s="5" t="inlineStr">
         <is>
           <t>Là quản trị hệ thống, tôi muốn huấn luyện lại và đo chất lượng mô hình xếp hạng gợi ý, để chất lượng đề xuất được cải thiện theo thời gian.</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr">
+      <c r="D70" s="5" t="inlineStr">
         <is>
           <t>- Quản trị viên kích hoạt được quá trình huấn luyện lại mô hình từ dữ liệu quan hệ và tương tác hiện có
 - Quá trình huấn luyện chạy nền, không làm gián đoạn việc phục vụ gợi ý cho người dùng
 - Sau khi huấn luyện, hệ thống trả về các chỉ số đánh giá để so sánh với phiên bản trước
 - Mô hình mới chỉ được đưa vào sử dụng khi chỉ số đánh giá không kém hơn mô hình đang chạy
-- Chỉ tài khoản có quyền quản trị mới kích hoạt được huấn luyện và đánh giá</t>
+- Chỉ tài khoản có quyền quản trị mới kích hoạt được huấn luyện và đánh giá
+- Kết quả huấn luyện và chỉ số đánh giá được ghi lại kèm mốc thời gian để so sánh giữa các lần
+- Yêu cầu huấn luyện gửi trùng khi tiến trình đang chạy sẽ bị từ chối kèm thông báo rõ ràng</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr">
@@ -2882,17 +3174,17 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="F70" s="5" t="inlineStr">
         <is>
           <t>Chất lượng gợi ý xuống cấp theo thời gian khi hành vi người dùng thay đổi. Chu trình huấn luyện và đánh giá có kiểm soát cho phép cải tiến liên tục mà không rủi ro làm xấu trải nghiệm.</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="141" customHeight="1">
-      <c r="A71" s="7" t="n">
+    <row r="71" ht="195" customHeight="1">
+      <c r="A71" s="8" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="8" t="inlineStr">
+      <c r="B71" s="9" t="inlineStr">
         <is>
           <t>Hoàn tất kết bạn trọn vẹn qua nhiều dịch vụ</t>
         </is>
@@ -2908,7 +3200,9 @@
 - Người dùng chỉ thấy kết quả khi cả ba phần đã hoàn tất, không thấy trạng thái nửa vời
 - Toàn bộ quá trình hoàn tất trong thời gian đủ ngắn để người dùng cảm nhận là tức thời
 - Nếu cùng một lời mời bị xử lý nhiều lần do lỗi mạng, hệ thống chỉ tạo một bộ dữ liệu duy nhất
-- Trạng thái xử lý được ghi lại để có thể truy vết khi cần kiểm tra</t>
+- Trạng thái xử lý được ghi lại để có thể truy vết khi cần kiểm tra
+- Trong lúc chờ hoàn tất, giao diện hiển thị trạng thái đang xử lý thay vì để nút im lặng không phản hồi
+- Nếu quá trình vượt thời gian chờ hợp lý, người dùng nhận thông báo đang xử lý và được hướng dẫn kiểm tra lại sau</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
@@ -2922,11 +3216,11 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="96" customHeight="1">
-      <c r="A72" s="7" t="n">
+    <row r="72" ht="165" customHeight="1">
+      <c r="A72" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="B72" s="8" t="inlineStr">
+      <c r="B72" s="9" t="inlineStr">
         <is>
           <t>Tự động hoàn tác khi một bước thất bại</t>
         </is>
@@ -2942,7 +3236,9 @@
 - Sau khi hoàn tác, người dùng có thể thử chấp nhận lại lời mời từ đầu
 - Hệ thống không để tồn tại quan hệ bạn bè thiếu cuộc trò chuyện hoặc ngược lại
 - Quá trình hoàn tác được ghi lại đầy đủ để đội vận hành kiểm tra khi cần
-- Hoàn tác lặp lại nhiều lần cũng cho ra cùng một kết quả cuối cùng</t>
+- Hoàn tác lặp lại nhiều lần cũng cho ra cùng một kết quả cuối cùng
+- Người dùng nhận thông báo lỗi diễn đạt theo ngôn ngữ đời thường, không lộ tên bước xử lý nội bộ
+- Sau khi hoàn tác, giao diện hai phía trở về đúng trạng thái trước khi thao tác, không còn dấu vết nửa vời</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
@@ -2956,11 +3252,11 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="111" customHeight="1">
-      <c r="A73" s="7" t="n">
+    <row r="73" ht="165" customHeight="1">
+      <c r="A73" s="8" t="n">
         <v>72</v>
       </c>
-      <c r="B73" s="8" t="inlineStr">
+      <c r="B73" s="9" t="inlineStr">
         <is>
           <t>Không mất sự kiện khi dịch vụ tạm gián đoạn</t>
         </is>
@@ -2976,7 +3272,9 @@
 - Khi dịch vụ đích tạm ngừng, sự kiện được giữ lại và gửi lại khi dịch vụ hoạt động trở lại
 - Cùng một sự kiện được xử lý nhiều lần cũng chỉ tạo ra một kết quả duy nhất
 - Sự kiện thất bại nhiều lần liên tiếp được tách ra để đội vận hành xử lý riêng
-- Người dùng không cần thao tác lại khi hệ thống tự phục hồi</t>
+- Người dùng không cần thao tác lại khi hệ thống tự phục hồi
+- Người dùng không thấy thông báo lỗi kỹ thuật khi hệ thống đang tự phục hồi ở phía sau
+- Sự kiện được xử lý lại không tạo thông báo trùng cho người dùng</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
@@ -2990,95 +3288,103 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="126" customHeight="1">
-      <c r="A74" s="2" t="n">
+    <row r="74" ht="225" customHeight="1">
+      <c r="A74" s="4" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="5" t="inlineStr">
         <is>
           <t>Truy cập toàn hệ thống qua một cổng duy nhất</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Là người dùng, tôi muốn ứng dụng hoạt động mượt mà như một hệ thống thống nhất, để tôi không cảm nhận được sự phức tạp bên trong.</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>- Mọi yêu cầu từ giao diện đều đi qua một địa chỉ duy nhất và được định tuyến tới đúng dịch vụ xử lý
 - Chính sách chia sẻ tài nguyên giữa các miền được cấu hình tập trung, giao diện không gặp lỗi bị chặn
 - Khi một dịch vụ nội bộ gặp sự cố, người dùng nhận thông báo lỗi thân thiện thay vì lỗi kỹ thuật thô
 - Địa chỉ và cấu trúc nội bộ của các dịch vụ không bị lộ ra bên ngoài
-- Kết nối thời gian thực cũng đi qua cùng lớp cổng và giữ được kết nối lâu dài</t>
-        </is>
-      </c>
-      <c r="E74" s="6" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
+- Kết nối thời gian thực cũng đi qua cùng lớp cổng và giữ được kết nối lâu dài
+- Lỗi từ dịch vụ nội bộ được quy đổi thành thông điệp tiếng Việt dễ hiểu trước khi hiển thị
+- Yêu cầu quá thời gian chờ được huỷ và báo lỗi thay vì để giao diện chờ vô hạn
+- Khi máy chủ không phản hồi, giao diện hiển thị trạng thái lỗi có nút thử lại thay vì màn hình trắng</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
         <is>
           <t>Một cổng vào duy nhất che giấu độ phức tạp của kiến trúc nhiều dịch vụ, đồng thời là nơi tập trung áp dụng các chính sách chung về bảo mật, giới hạn tốc độ và ghi nhật ký.</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="156" customHeight="1">
-      <c r="A75" s="2" t="n">
+    <row r="75" ht="240" customHeight="1">
+      <c r="A75" s="4" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>Chặn truy cập khi chưa đăng nhập</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>Là quản trị hệ thống, tôi muốn mọi tài nguyên riêng tư đều yêu cầu phiên hợp lệ, để dữ liệu người dùng không bị truy cập trái phép.</t>
         </is>
       </c>
-      <c r="D75" s="4" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>- Truy cập bất kỳ trang nội bộ nào khi chưa đăng nhập đều bị chuyển về màn hình đăng nhập
 - Mọi yêu cầu dữ liệu không kèm phiên hợp lệ đều bị từ chối ở phía máy chủ, không chỉ ẩn ở giao diện
 - Các luồng công khai như đăng ký, đăng nhập và xác thực mã được khai báo rõ ràng thay vì mở mặc định
 - Kết nối thời gian thực cũng phải xác thực trước khi tham gia bất kỳ cuộc trò chuyện nào
-- Người dùng đã đăng nhập chỉ truy cập được dữ liệu mà mình có quyền, không phải toàn bộ dữ liệu hệ thống</t>
-        </is>
-      </c>
-      <c r="E75" s="5" t="inlineStr">
+- Người dùng đã đăng nhập chỉ truy cập được dữ liệu mà mình có quyền, không phải toàn bộ dữ liệu hệ thống
+- Người dùng bị chuyển về đăng nhập vẫn được đưa trở lại đúng trang định vào sau khi đăng nhập thành công
+- Trong lúc kiểm tra phiên, giao diện hiển thị trạng thái chờ thay vì nháy qua màn hình đăng nhập
+- Thông tin phiên và dữ liệu người dùng không bị ghi vào nhật ký trình duyệt hay lộ trong thông báo lỗi</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F75" s="4" t="inlineStr">
+      <c r="F75" s="5" t="inlineStr">
         <is>
           <t>Kiểm soát truy cập phải thực thi ở máy chủ vì giao diện có thể bị vượt qua. Nguyên tắc chặn mặc định và mở có chọn lọc giảm nguy cơ bỏ sót khi thêm tính năng mới.</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="141" customHeight="1">
-      <c r="A76" s="2" t="n">
+    <row r="76" ht="195" customHeight="1">
+      <c r="A76" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>Triển khai tự động khi có thay đổi mã nguồn</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>Là đội phát triển, chúng tôi muốn hệ thống tự động xây dựng và triển khai khi mã nguồn thay đổi, để tính năng mới tới tay người dùng nhanh và ít rủi ro.</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>- Khi mã nguồn được đưa lên nhánh chính, quy trình tự động xây dựng và triển khai được kích hoạt
 - Phần máy chủ được đóng gói, đẩy lên kho hình ảnh và cập nhật trên máy chủ chạy thật
 - Phần giao diện được xây dựng, đồng bộ lên kho tĩnh và làm mới bộ nhớ đệm phân phối nội dung
 - Đội phát triển kích hoạt được quy trình triển khai thủ công khi cần
-- Quy trình thất bại ở bất kỳ bước nào cũng dừng lại và không triển khai bản lỗi lên môi trường thật</t>
+- Quy trình thất bại ở bất kỳ bước nào cũng dừng lại và không triển khai bản lỗi lên môi trường thật
+- Quy trình chạy kiểm tra biên dịch và kiểm tra chất lượng mã trước khi đóng gói, lỗi ở bước này chặn triển khai
+- Kết quả từng lần chạy được ghi lại đủ để truy vết phiên bản nào đang chạy trên môi trường thật</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
@@ -3086,20 +3392,538 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="F76" s="5" t="inlineStr">
         <is>
           <t>Triển khai thủ công là nguồn sai sót và làm chậm nhịp phát hành. Tự động hoá toàn bộ chuỗi giúp thay đổi nhỏ được đưa ra thường xuyên, giảm rủi ro của mỗi lần phát hành.</t>
         </is>
       </c>
     </row>
+    <row r="77" ht="195" customHeight="1">
+      <c r="A77" s="17" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Hiển thị lỗi nhất quán toàn ứng dụng</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng, tôi muốn mọi lỗi đều được báo bằng ngôn ngữ dễ hiểu và đúng chỗ, để tôi biết chuyện gì đã xảy ra và phải làm gì tiếp theo.</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>- Lỗi của một ô nhập liệu hiển thị ngay dưới ô đó; lỗi của cả biểu mẫu hiển thị cố định trên biểu mẫu; chỉ lỗi của thao tác nền mới dùng thông báo nổi
+- Không có màn hình nào hiển thị mã lỗi kỹ thuật, tên ngoại lệ hay vết gọi hàm cho người dùng cuối
+- Mọi lỗi có thể thử lại đều đi kèm nút thử lại đặt ngay tại khu vực bị lỗi, không bắt người dùng tải lại cả trang
+- Mất kết nối mạng và máy chủ trả lỗi được phân biệt bằng hai thông điệp khác nhau
+- Cùng một lỗi lặp lại nhiều lần chỉ hiển thị một thông báo, không xếp chồng nhiều thông báo giống hệt nhau
+- Lỗi khiến toàn bộ giao diện sập được bắt lại bởi lớp bảo vệ chung, hiển thị màn hình lỗi có nút tải lại thay vì trang trắng
+- Thông báo lỗi được trình đọc màn hình đọc lên ngay khi xuất hiện</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Ứng dụng hiện đã có sẵn hàm trích thông điệp lỗi và thông báo nổi, nhưng cách dùng chưa thống nhất giữa các màn hình: có nơi chỉ hiện thông báo nổi rồi tự tắt, có nơi im lặng. US này chuẩn hoá quy ước hiển thị lỗi để người dùng luôn hiểu và luôn có đường thoát.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="180" customHeight="1">
+      <c r="A78" s="18" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>Trạng thái tải và trạng thái rỗng nhất quán</t>
+        </is>
+      </c>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>Là người dùng, tôi muốn biết ứng dụng đang tải hay thực sự không có dữ liệu, để không nhầm màn hình trống là lỗi.</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>- Mọi danh sách và bảng đều hiển thị khung xương đúng bố cục thật trong lần tải đầu, không dùng màn hình trắng hay ô chữ đang tải
+- Khung xương giữ đúng chiều cao của nội dung thật để bố cục không nhảy khi dữ liệu về
+- Mọi trạng thái rỗng gồm ba phần: điều gì chưa có, vì sao điều đó bình thường, và một hành động tiếp theo rõ ràng
+- Trạng thái rỗng do lọc hoặc tìm kiếm khác với trạng thái rỗng do chưa có dữ liệu nào
+- Mọi nút gây ra thao tác mạng đều có trạng thái đang xử lý và bị vô hiệu trong lúc chờ
+- Trạng thái đang tải được thông báo cho trình đọc màn hình bằng nhãn mô tả đang tải cái gì</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F78" s="9" t="inlineStr">
+        <is>
+          <t>Dự án đã có sẵn bộ ba thành phần khung xương, chỉ báo tải và trạng thái rỗng. US này biến chúng thành ràng buộc bắt buộc cho mọi màn hình, thay vì tuỳ nơi dùng nơi không.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="255" customHeight="1">
+      <c r="A79" s="17" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Phân trang và tải thêm đúng chuẩn</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng có nhiều dữ liệu, tôi muốn danh sách tải theo từng phần một cách đáng tin cậy, để không bị trùng, thiếu hay treo màn hình.</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>- Danh sách có dữ liệu thay đổi liên tục dùng phân trang theo con trỏ; danh sách tĩnh dùng phân trang theo số trang; mỗi màn hình khai báo rõ mình dùng loại nào
+- Con trỏ phân trang xử lý được các bản ghi có cùng mốc thời gian bằng cách kèm thêm định danh, không lặp lại hay bỏ sót bản ghi
+- Cuộn nhanh hoặc bấm liên tục không kích hoạt nhiều lần tải chồng nhau cho cùng một trang
+- Bản ghi mới chèn vào đầu danh sách trong lúc đang tải thêm không làm lệch các trang sau
+- Đã tải hết dữ liệu thì giao diện nói rõ đã hết và không còn kích hoạt tải thêm
+- Tải thêm thất bại thì hiển thị lỗi kèm nút thử lại tại cuối danh sách và giữ nguyên phần đã tải
+- Vị trí cuộn được giữ nguyên sau mỗi lần tải thêm, kể cả khi tải thêm về phía đầu danh sách
+- Kích thước trang được thống nhất theo từng loại danh sách thay vì mỗi màn hình tự chọn một con số khác nhau</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Hiện tại mỗi danh sách trong ứng dụng đang tự chọn cách phân trang và kích thước trang riêng: thông báo dùng số trang cỡ mười, bạn bè tải một trăm bản ghi một lần, hội thoại và tin nhắn dùng con trỏ. US này đặt ra chuẩn chung và các bẫy phải tránh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="120" customHeight="1">
+      <c r="A80" s="18" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="9" t="inlineStr">
+        <is>
+          <t>Số đếm chưa đọc chính xác</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>Là người dùng, tôi muốn các con số chưa đọc trên chuông và trên danh sách luôn đúng, để tôi tin được vào chúng.</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>- Số chưa đọc luôn lấy từ máy chủ, không suy ra từ số bản ghi đã tải về ở phía trình duyệt
+- Số chưa đọc vẫn đúng khi tổng số vượt quá kích thước một trang dữ liệu
+- Số đếm được đồng bộ lại sau khi kết nối thời gian thực khôi phục hoặc khi tải lại trang
+- Số đếm giảm ngay khi người dùng đọc và không bật trở lại giá trị cũ sau đó
+- Số vượt ngưỡng hiển thị được rút gọn nhưng nhãn dành cho trình đọc màn hình vẫn nêu con số đầy đủ</t>
+        </is>
+      </c>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>Huy hiệu chuông thông báo hiện đang đếm từ mảng thông báo đã tải về trình duyệt, trong khi mỗi lần chỉ tải mười bản ghi — nghĩa là người có nhiều hơn mười thông báo chưa đọc sẽ thấy con số sai. Máy chủ đã có sẵn điểm truy cập trả về số chưa đọc; US này yêu cầu giao diện dùng đúng nguồn số liệu đó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="180" customHeight="1">
+      <c r="A81" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Xác nhận trước thao tác không hoàn tác được</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng, tôi muốn được hỏi lại trước những thao tác không thể lấy lại, để một cú bấm nhầm không xoá mất dữ liệu của tôi.</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>- Mọi thao tác xoá, thu hồi, rời nhóm và đóng bình chọn đều hỏi xác nhận nêu rõ hậu quả cụ thể
+- Hộp thoại xác nhận nêu đích danh đối tượng bị tác động, không dùng câu hỏi chung chung
+- Nút xác nhận của thao tác phá huỷ dùng kiểu cảnh báo và không phải nút được chọn sẵn
+- Hộp thoại đóng được bằng phím Esc, tiêu điểm bị giữ trong hộp thoại và trả về đúng chỗ cũ khi đóng
+- Trong lúc thực hiện, nút xác nhận hiển thị trạng thái đang xử lý và chặn bấm lặp
+- Thao tác thất bại thì trạng thái được hoàn nguyên nguyên vẹn kèm thông báo lý do</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Nhiều thao tác phá huỷ trong ứng dụng đang thực hiện ngay khi bấm. US này chuẩn hoá một mẫu xác nhận dùng chung cho tất cả, thay vì mỗi màn hình tự nghĩ ra một cách hỏi khác nhau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="210" customHeight="1">
+      <c r="A82" s="18" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
+        <is>
+          <t>Sử dụng được bằng bàn phím và trình đọc màn hình</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>Là người dùng không dùng chuột hoặc dùng trình đọc màn hình, tôi muốn thao tác được mọi chức năng chính, để ứng dụng không loại trừ tôi.</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>- Mọi thao tác chính đều thực hiện được chỉ bằng bàn phím: đăng nhập, tìm người, kết bạn, mở cuộc trò chuyện, gửi tin nhắn, mở thông báo
+- Thứ tự di chuyển bằng phím Tab đi theo đúng thứ tự thị giác, không nhảy cóc và không rơi vào phần tử bị ẩn
+- Mọi phần tử nhận tiêu điểm đều có vòng tiêu điểm nhìn thấy rõ trên cả nền sáng lẫn nền tối
+- Hộp thoại và bảng trượt giữ tiêu điểm bên trong khi mở, đóng bằng phím Esc và trả tiêu điểm về phần tử đã kích hoạt
+- Mọi nút chỉ có biểu tượng đều có nhãn chữ dành cho trình đọc màn hình
+- Thông tin không bao giờ chỉ được truyền tải bằng màu sắc; luôn có thêm hình dạng, biểu tượng hoặc chữ đi kèm
+- Có liên kết bỏ qua phần điều hướng để đi thẳng vào nội dung chính
+- Tin nhắn mới đến và thông báo lỗi được công bố qua vùng thông báo động cho trình đọc màn hình</t>
+        </is>
+      </c>
+      <c r="E82" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F82" s="9" t="inlineStr">
+        <is>
+          <t>Đợt làm lại giao diện trước đã dựng nền tảng về tương phản màu và một kiểu vòng tiêu điểm dùng chung. US này bổ sung phần còn thiếu: điều hướng bằng bàn phím, quản lý tiêu điểm trong hộp thoại và nhãn cho trình đọc màn hình.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="210" customHeight="1">
+      <c r="A83" s="17" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Dùng tốt trên màn hình nhỏ</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng dùng điện thoại hoặc cửa sổ hẹp, tôi muốn mọi màn hình vẫn dùng được, để không phải chuyển sang máy tính mới làm được việc.</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>- Không màn hình nào sinh thanh cuộn ngang ở chiều rộng ba trăm sáu mươi điểm ảnh
+- Bố cục ba cột của trang trò chuyện chuyển thành từng lớp riêng trên màn hình hẹp, có đường quay lại rõ ràng
+- Bảng thông tin cuộc trò chuyện và các bảng phụ hiển thị dạng lớp phủ toàn màn hình thay vì cột bị bóp lại
+- Ô soạn tin và thanh công cụ luôn nằm trong tầm với, không bị bàn phím ảo che mất
+- Mọi vùng bấm trên thiết bị cảm ứng đạt kích thước tối thiểu bốn mươi bốn điểm ảnh
+- Bảng và danh sách rộng cuộn ngang trong khung riêng của chúng, không đẩy cả trang trôi ngang
+- Nội dung dài và chuỗi ký tự liền không dấu cách luôn xuống dòng thay vì làm vỡ bố cục</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Ứng dụng hiện được thiết kế theo hướng ưu tiên máy tính. US này đặt ra ràng buộc tối thiểu để các màn hình chính vẫn dùng được trên điện thoại mà không phải viết lại giao diện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="180" customHeight="1">
+      <c r="A84" s="18" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="9" t="inlineStr">
+        <is>
+          <t>Phản hồi khi mất kết nối thời gian thực</t>
+        </is>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>Là người dùng đang trò chuyện, tôi muốn biết khi nào mình mất kết nối và khi nào đã nối lại, để không hiểu nhầm là mọi người đột nhiên im lặng.</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>- Mất kết nối quá một khoảng ngắn thì hiển thị dải thông báo rõ ràng ở đầu ứng dụng
+- Ứng dụng tự kết nối lại theo khoảng chờ tăng dần thay vì thử liên tục gây quá tải
+- Kết nối lại thành công thì dải thông báo tự ẩn và ứng dụng đồng bộ lại tin nhắn, số chưa đọc và trạng thái trực tuyến bị bỏ lỡ
+- Trong lúc mất kết nối, nút gửi tin nhắn vẫn dùng được và tin nhắn được xếp hàng chờ thay vì bị chặn
+- Trạng thái đang gõ và trạng thái trực tuyến cũ bị xoá khi mất kết nối, không hiển thị thông tin đã lỗi thời
+- Dải thông báo không che mất nội dung hay đẩy bố cục nhảy khi xuất hiện và biến mất</t>
+        </is>
+      </c>
+      <c r="E84" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="inlineStr">
+        <is>
+          <t>Ứng dụng dựa nhiều vào kênh thời gian thực nhưng chưa cho người dùng biết khi kênh đó đứt. US này lấp khoảng trống giữa việc mất kết nối và việc người dùng nhận ra điều đó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="135" customHeight="1">
+      <c r="A85" s="17" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Chống thao tác lặp và gửi trùng</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng hay bấm nhanh hoặc mạng chậm, tôi muốn một thao tác chỉ tạo ra đúng một kết quả, để không sinh dữ liệu trùng.</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>- Mọi nút gửi biểu mẫu bị vô hiệu trong lúc yêu cầu đang chạy và chỉ bật lại khi có kết quả
+- Các thao tác tạo dữ liệu mang mã do máy khách sinh ra để máy chủ nhận ra và bỏ qua yêu cầu trùng
+- Ô tìm kiếm và các ô lọc chờ người dùng ngừng gõ rồi mới gọi máy chủ
+- Kết quả của yêu cầu cũ về sau kết quả mới thì bị bỏ qua, giao diện luôn khớp với thao tác gần nhất
+- Rời khỏi màn hình sẽ huỷ các yêu cầu đang chạy của màn hình đó, không cập nhật vào giao diện đã đóng</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Ứng dụng đã áp dụng mã tin nhắn do máy khách sinh cho luồng gửi tin nhắn. US này mở rộng cùng nguyên tắc sang các thao tác tạo dữ liệu khác như tạo nhóm, gửi lời mời kết bạn và tạo bình chọn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="120" customHeight="1">
+      <c r="A86" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="9" t="inlineStr">
+        <is>
+          <t>Giới hạn tần suất cho thao tác nhạy cảm</t>
+        </is>
+      </c>
+      <c r="C86" s="9" t="inlineStr">
+        <is>
+          <t>Là quản trị hệ thống, tôi muốn các thao tác dễ bị lạm dụng đều có giới hạn tần suất, để bảo vệ người dùng và chi phí vận hành.</t>
+        </is>
+      </c>
+      <c r="D86" s="9" t="inlineStr">
+        <is>
+          <t>- Đăng nhập, đăng ký, gửi lại mã và gửi lời mời kết bạn đều có giới hạn số lần trong một khoảng thời gian
+- Vượt giới hạn thì máy chủ trả về mã trạng thái đúng chuẩn kèm thông tin thời gian phải chờ
+- Giao diện hiển thị thời gian chờ còn lại thay vì thông báo lỗi chung chung
+- Giới hạn được áp ở phía máy chủ, không chỉ vô hiệu nút ở phía trình duyệt
+- Người dùng hợp lệ trong quá trình sử dụng bình thường không bao giờ chạm phải giới hạn này</t>
+        </is>
+      </c>
+      <c r="E86" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F86" s="9" t="inlineStr">
+        <is>
+          <t>Bản thân các tiêu chí về khoảng chờ gửi lại mã đã ngụ ý phải có giới hạn tần suất. US này nêu rõ yêu cầu đó thành một điều kiện kiểm thử được, cho cả phía máy chủ lẫn cách giao diện phản hồi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="180" customHeight="1">
+      <c r="A87" s="17" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Hiển thị thời gian, số và tên nhất quán</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng Việt Nam, tôi muốn mọi mốc thời gian, con số và tên hiển thị theo cùng một quy ước, để đọc lướt vẫn hiểu ngay.</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>- Mốc thời gian trong vòng một ngày hiển thị dạng tương đối; xa hơn hiển thị dạng ngày tháng đầy đủ theo quy ước Việt Nam
+- Mọi mốc thời gian rút gọn đều có thời điểm đầy đủ khi di chuột hoặc chạm giữ
+- Mốc thời gian tương đối tự cập nhật theo thời gian thực mà không cần tải lại trang
+- Dung lượng tệp và các con số lớn hiển thị theo đơn vị dễ đọc, có phân cách hàng nghìn
+- Tên hiển thị quá dài bị cắt bằng dấu ba chấm ở cùng một ngưỡng trên mọi màn hình và hiển thị đầy đủ khi di chuột
+- Người dùng chưa đặt tên hiển thị thì mọi màn hình cùng dùng một giá trị thay thế thống nhất</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Ứng dụng đã có sẵn các hàm định dạng thời gian. US này yêu cầu dùng chúng ở mọi nơi thay vì để một số màn hình tự dựng chuỗi thời gian riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="150" customHeight="1">
+      <c r="A88" s="18" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="9" t="inlineStr">
+        <is>
+          <t>Bảo vệ dữ liệu người dùng trên trình duyệt</t>
+        </is>
+      </c>
+      <c r="C88" s="9" t="inlineStr">
+        <is>
+          <t>Là người dùng dùng máy tính chung, tôi muốn dữ liệu của mình không sót lại trên trình duyệt, để người dùng sau không đọc được.</t>
+        </is>
+      </c>
+      <c r="D88" s="9" t="inlineStr">
+        <is>
+          <t>- Đăng xuất xoá sạch toàn bộ kho lưu trữ cục bộ và bộ nhớ tạm của ứng dụng, kể cả phần được lưu bền
+- Đăng nhập bằng tài khoản khác không bao giờ hiển thị dữ liệu còn sót của tài khoản trước
+- Nội dung tin nhắn, email và thông tin phiên không bao giờ được ghi ra bảng điều khiển của trình duyệt ở bản dựng thật
+- Địa chỉ trên thanh URL không chứa thông tin nhạy cảm như mã xác thực hay email
+- Dữ liệu lưu bền trên trình duyệt chỉ gồm phần cần thiết cho trải nghiệm, không gồm thông tin định danh nhạy cảm</t>
+        </is>
+      </c>
+      <c r="E88" s="11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F88" s="9" t="inlineStr">
+        <is>
+          <t>Ứng dụng lưu trạng thái xuống trình duyệt để giữ phiên qua các lần tải lại. US này đặt ra ranh giới cho việc lưu cái gì và bắt buộc phải dọn sạch những gì khi đăng xuất.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="150" customHeight="1">
+      <c r="A89" s="17" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Tốc độ tải và phản hồi của giao diện</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng, tôi muốn ứng dụng mở nhanh và phản hồi tức thì, để việc trò chuyện không bị ngắt quãng vì phải chờ.</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>- Màn hình đăng nhập và màn hình trò chuyện hiển thị nội dung đầu tiên trong vòng hai giây trên kết nối bình thường
+- Các trang phụ được tải theo nhu cầu, không dồn hết vào gói tải ban đầu
+- Mọi thao tác của người dùng có phản hồi thị giác trong vòng một trăm mili giây, kể cả khi kết quả thật còn phải chờ máy chủ
+- Danh sách dài không dựng lại toàn bộ khi chỉ một phần tử thay đổi
+- Ảnh và video chỉ tải khi cuộn tới và luôn có chỗ dành sẵn để bố cục không nhảy
+- Chuyển đổi giữa các cuộc trò chuyện hiển thị nội dung đã có trong bộ nhớ ngay, phần thiếu tải bổ sung ở phía sau</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Ứng dụng dùng công cụ đóng gói có sẵn khả năng phân tích kích thước gói. US này chuyển các mong đợi về tốc độ thành ngưỡng cụ thể có thể đo được thay vì cảm tính.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="150" customHeight="1">
+      <c r="A90" s="18" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="9" t="inlineStr">
+        <is>
+          <t>Giữ nguyên trạng thái làm việc khi tải lại</t>
+        </is>
+      </c>
+      <c r="C90" s="9" t="inlineStr">
+        <is>
+          <t>Là người dùng lỡ tải lại trang hoặc mở lại đường dẫn, tôi muốn quay về đúng chỗ mình đang làm, để không phải thao tác lại từ đầu.</t>
+        </is>
+      </c>
+      <c r="D90" s="9" t="inlineStr">
+        <is>
+          <t>- Đường dẫn trên trình duyệt phản ánh đúng cuộc trò chuyện, tab và bộ lọc đang mở
+- Nút quay lại và tiến tới của trình duyệt hoạt động đúng trên mọi màn hình, không đưa người dùng ra khỏi ứng dụng ngoài ý muốn
+- Nội dung đang soạn dở của từng cuộc trò chuyện được giữ lại khi chuyển qua lại giữa các cuộc trò chuyện
+- Tải lại trang trong lúc đang mở một cuộc trò chuyện sẽ trở lại đúng cuộc trò chuyện đó
+- Mở đường dẫn tới cuộc trò chuyện không tồn tại hoặc không có quyền thì hiển thị thông báo rõ ràng thay vì màn hình trống</t>
+        </is>
+      </c>
+      <c r="E90" s="11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F90" s="9" t="inlineStr">
+        <is>
+          <t>Ứng dụng đã có đường dẫn riêng cho từng cuộc trò chuyện. US này mở rộng nguyên tắc đó sang các trạng thái giao diện khác để đường dẫn luôn là nguồn sự thật.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="120" customHeight="1">
+      <c r="A91" s="17" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Giao diện sáng tối và tuỳ chọn hiển thị</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Là người dùng làm việc buổi tối hoặc nhạy cảm với chuyển động, tôi muốn giao diện tôn trọng thiết lập của tôi, để dùng lâu không mỏi mắt.</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>- Lựa chọn sáng, tối và theo hệ thống đều hoạt động đúng và được ghi nhớ giữa các phiên
+- Không có màn hình nào bị loá trắng trong khoảnh khắc khi tải ở chế độ tối
+- Mọi cặp màu chữ trên nền đạt ngưỡng tương phản tối thiểu ở cả hai chế độ
+- Khi hệ thống bật chế độ giảm chuyển động, mọi hiệu ứng chuyển cảnh và động bị tắt và hiển thị thẳng trạng thái cuối
+- Trạng thái đọc được ở chế độ tối lẫn sáng mà không phụ thuộc vào việc phân biệt màu</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Đợt làm lại giao diện trước đã kiểm chứng tương phản màu bằng công cụ tính toán. US này biến các kết quả đó thành tiêu chí nghiệm thu để những thay đổi sau này không làm hỏng chúng.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F76"/>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"P1,P2,P3"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>